<commit_message>
2021-05-07 End of day file push
</commit_message>
<xml_diff>
--- a/Tax/calcs.xlsx
+++ b/Tax/calcs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABriggs\Documents\BWS\Tax\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC229228-677A-40FD-813E-B03343AEBF8F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD5F9C2-3090-4D77-8CDC-56D98DCCA050}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3945" yWindow="1065" windowWidth="21600" windowHeight="11385" xr2:uid="{6D0CD4EE-CC56-4F74-B7F8-52D61ECC5DE1}"/>
   </bookViews>
@@ -132,12 +132,19 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;\ #,##0_)&quot;/ Hr&quot;;\(&quot;$&quot;\ #,##0\)&quot;/ Hr&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;\ #,##0_)&quot;/ Hr&quot;;\(&quot;$&quot;\ #,##0\)&quot;/ Hr&quot;"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -536,7 +543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -553,9 +560,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -581,9 +585,6 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -601,15 +602,21 @@
     <xf numFmtId="164" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
@@ -621,28 +628,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -653,9 +678,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF5D5D"/>
       <color rgb="FF4D55FF"/>
       <color rgb="FF4DFF4D"/>
-      <color rgb="FFFF5D5D"/>
       <color rgb="FF2FFAFF"/>
       <color rgb="FFFE48E4"/>
       <color rgb="FFFEF254"/>
@@ -989,32 +1014,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C1" s="67" t="s">
+      <c r="C1" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="57">
+      <c r="D1" s="58"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="55">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C2" s="67" t="s">
+      <c r="C2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="67"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="57">
+      <c r="D2" s="58"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="55">
         <v>48</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="56">
+      <c r="D3" s="58"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="54">
         <v>231</v>
       </c>
     </row>
@@ -1023,46 +1048,46 @@
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="66"/>
+      <c r="D5" s="61"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
       <c r="F6">
         <f>($F$3) * F1 * 60 * 60</f>
         <v>6652800</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C7" s="66" t="s">
+      <c r="C7" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="66"/>
-      <c r="E7" s="66"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
       <c r="F7">
         <f>($F$3) * F1 * 60</f>
         <v>110880</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="66"/>
-      <c r="E8" s="66"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
       <c r="F8">
         <f>($F$3) * F1</f>
         <v>1848</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="14" t="s">
         <v>23</v>
       </c>
       <c r="G11" t="s">
@@ -1070,11 +1095,11 @@
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C12" s="71" t="s">
+      <c r="C12" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="72"/>
-      <c r="E12" s="57">
+      <c r="D12" s="69"/>
+      <c r="E12" s="55">
         <v>42000</v>
       </c>
       <c r="F12" t="s">
@@ -1092,19 +1117,19 @@
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C13" s="71" t="s">
+      <c r="C13" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="72"/>
-      <c r="E13" s="56">
-        <v>95000</v>
+      <c r="D13" s="71"/>
+      <c r="E13" s="54">
+        <v>56375</v>
       </c>
       <c r="F13" t="s">
         <v>20</v>
       </c>
       <c r="G13">
         <f>E13</f>
-        <v>95000</v>
+        <v>56375</v>
       </c>
       <c r="H13" t="s">
         <v>20</v>
@@ -1115,11 +1140,11 @@
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="58"/>
-      <c r="E14" s="56">
+      <c r="D14" s="73"/>
+      <c r="E14" s="54">
         <v>100</v>
       </c>
       <c r="F14" t="s">
@@ -1151,15 +1176,15 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
-      <c r="I16" s="70"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58"/>
+      <c r="H16" s="58"/>
+      <c r="I16" s="59"/>
       <c r="J16" s="63" t="s">
         <v>17</v>
       </c>
@@ -1211,355 +1236,355 @@
       <c r="P17" s="6"/>
     </row>
     <row r="18" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="40">
-        <f>E12</f>
+      <c r="B18" s="77">
+        <f>$E$12</f>
         <v>42000</v>
       </c>
-      <c r="C18" s="16">
+      <c r="C18" s="15">
         <f>(((($E$12/365)/24)/60)/60)</f>
         <v>1.3318112633181126E-3</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="16">
         <f>((($E$12/365)/24)/60)</f>
         <v>7.9908675799086754E-2</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <f>(($E$12/365)/24)</f>
         <v>4.7945205479452051</v>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="18">
         <f>($E$12/365)</f>
         <v>115.06849315068493</v>
       </c>
-      <c r="G18" s="17">
+      <c r="G18" s="16">
         <f>($E$12/52)</f>
         <v>807.69230769230774</v>
       </c>
-      <c r="H18" s="17">
+      <c r="H18" s="16">
         <f>($E$12/12)</f>
         <v>3500</v>
       </c>
-      <c r="I18" s="20">
+      <c r="I18" s="19">
         <f>($E$12/4)</f>
         <v>10500</v>
       </c>
-      <c r="J18" s="21">
+      <c r="J18" s="20">
         <f>$E$12/$F$6</f>
         <v>6.313131313131313E-3</v>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="21">
         <f>$E$12/$F$7</f>
         <v>0.37878787878787878</v>
       </c>
-      <c r="L18" s="19">
+      <c r="L18" s="18">
         <f>$E$12/$F$8</f>
         <v>22.727272727272727</v>
       </c>
-      <c r="M18" s="22">
+      <c r="M18" s="21">
         <f>$E$12/$F$3</f>
         <v>181.81818181818181</v>
       </c>
-      <c r="N18" s="23">
+      <c r="N18" s="22">
         <f>$E$12/$F$2</f>
         <v>875</v>
       </c>
       <c r="O18" s="7"/>
     </row>
     <row r="19" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="40">
-        <f>E13</f>
-        <v>95000</v>
-      </c>
-      <c r="C19" s="24">
+      <c r="B19" s="75">
+        <f>$E$13</f>
+        <v>56375</v>
+      </c>
+      <c r="C19" s="23">
         <f>(((($E$13/365)/24)/60)/60)</f>
-        <v>3.012430238457636E-3</v>
-      </c>
-      <c r="D19" s="25">
+        <v>1.7876395230847285E-3</v>
+      </c>
+      <c r="D19" s="24">
         <f>((($E$13/365)/24)/60)</f>
-        <v>0.18074581430745815</v>
-      </c>
-      <c r="E19" s="26">
+        <v>0.10725837138508371</v>
+      </c>
+      <c r="E19" s="25">
         <f>(($E$13/365)/24)</f>
-        <v>10.844748858447488</v>
-      </c>
-      <c r="F19" s="27">
+        <v>6.4355022831050226</v>
+      </c>
+      <c r="F19" s="26">
         <f>($E$13/365)</f>
-        <v>260.27397260273972</v>
-      </c>
-      <c r="G19" s="25">
+        <v>154.45205479452054</v>
+      </c>
+      <c r="G19" s="24">
         <f>($E$13/52)</f>
-        <v>1826.9230769230769</v>
-      </c>
-      <c r="H19" s="25">
+        <v>1084.1346153846155</v>
+      </c>
+      <c r="H19" s="24">
         <f>($E$13/12)</f>
-        <v>7916.666666666667</v>
-      </c>
-      <c r="I19" s="28">
+        <v>4697.916666666667</v>
+      </c>
+      <c r="I19" s="27">
         <f>($E$13/4)</f>
-        <v>23750</v>
-      </c>
-      <c r="J19" s="29">
+        <v>14093.75</v>
+      </c>
+      <c r="J19" s="28">
         <f>$E$13/$F$6</f>
-        <v>1.4279701779701779E-2</v>
-      </c>
-      <c r="K19" s="30">
+        <v>8.4738756613756613E-3</v>
+      </c>
+      <c r="K19" s="29">
         <f>$E$13/$F$7</f>
-        <v>0.85678210678210676</v>
-      </c>
-      <c r="L19" s="27">
+        <v>0.50843253968253965</v>
+      </c>
+      <c r="L19" s="26">
         <f>$E$13/$F$8</f>
-        <v>51.406926406926409</v>
-      </c>
-      <c r="M19" s="30">
+        <v>30.50595238095238</v>
+      </c>
+      <c r="M19" s="29">
         <f>$E$13/$F$3</f>
-        <v>411.25541125541127</v>
-      </c>
-      <c r="N19" s="31">
+        <v>244.04761904761904</v>
+      </c>
+      <c r="N19" s="30">
         <f>$E$13/$F$2</f>
-        <v>1979.1666666666667</v>
+        <v>1174.4791666666667</v>
       </c>
       <c r="O19" s="7"/>
     </row>
     <row r="20" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="73">
-        <f>E14</f>
+      <c r="B20" s="79">
+        <f>$E$14</f>
         <v>100</v>
       </c>
-      <c r="C20" s="32">
+      <c r="C20" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60)</f>
         <v>5.8599695585996965E-3</v>
       </c>
-      <c r="D20" s="33">
+      <c r="D20" s="32">
         <f>$G$14/365 / 24 / 60</f>
         <v>0.35159817351598177</v>
       </c>
-      <c r="E20" s="33">
+      <c r="E20" s="32">
         <f>$G$14/365/24</f>
         <v>21.095890410958905</v>
       </c>
-      <c r="F20" s="34">
+      <c r="F20" s="33">
         <f>$G$14 / 365</f>
         <v>506.30136986301369</v>
       </c>
-      <c r="G20" s="33">
+      <c r="G20" s="32">
         <f>$G$14 / 52</f>
         <v>3553.8461538461538</v>
       </c>
-      <c r="H20" s="33">
+      <c r="H20" s="32">
         <f>$G$14/12</f>
         <v>15400</v>
       </c>
-      <c r="I20" s="35">
+      <c r="I20" s="34">
         <f>$G$14/4</f>
         <v>46200</v>
       </c>
-      <c r="J20" s="36">
+      <c r="J20" s="35">
         <f>(($E$14 / 60) / 60)</f>
         <v>2.777777777777778E-2</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="33">
         <f>$E$14/60</f>
         <v>1.6666666666666667</v>
       </c>
-      <c r="L20" s="37">
+      <c r="L20" s="36">
         <f>$E$14</f>
         <v>100</v>
       </c>
-      <c r="M20" s="38">
+      <c r="M20" s="37">
         <f>$E$14*$F$1</f>
         <v>800</v>
       </c>
-      <c r="N20" s="34">
+      <c r="N20" s="33">
         <f>$E$14*$F$1*5</f>
         <v>4000</v>
       </c>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="39">
+      <c r="B21" s="77"/>
+      <c r="C21" s="38">
         <f>C19-C18</f>
-        <v>1.6806189751395234E-3</v>
-      </c>
-      <c r="D21" s="46">
+        <v>4.5582825976661591E-4</v>
+      </c>
+      <c r="D21" s="44">
         <f t="shared" ref="D21:N21" si="0">D19-D18</f>
-        <v>0.10083713850837139</v>
-      </c>
-      <c r="E21" s="50">
+        <v>2.7349695585996953E-2</v>
+      </c>
+      <c r="E21" s="48">
         <f t="shared" si="0"/>
-        <v>6.0502283105022832</v>
-      </c>
-      <c r="F21" s="50">
+        <v>1.6409817351598175</v>
+      </c>
+      <c r="F21" s="48">
         <f t="shared" si="0"/>
-        <v>145.20547945205479</v>
-      </c>
-      <c r="G21" s="54">
+        <v>39.383561643835606</v>
+      </c>
+      <c r="G21" s="52">
         <f t="shared" si="0"/>
-        <v>1019.2307692307692</v>
-      </c>
-      <c r="H21" s="46">
+        <v>276.44230769230774</v>
+      </c>
+      <c r="H21" s="44">
         <f>H19-H18</f>
-        <v>4416.666666666667</v>
-      </c>
-      <c r="I21" s="47">
+        <v>1197.916666666667</v>
+      </c>
+      <c r="I21" s="45">
         <f t="shared" si="0"/>
-        <v>13250</v>
-      </c>
-      <c r="J21" s="39">
+        <v>3593.75</v>
+      </c>
+      <c r="J21" s="38">
         <f t="shared" si="0"/>
-        <v>7.9665704665704655E-3</v>
-      </c>
-      <c r="K21" s="41">
+        <v>2.1607443482443483E-3</v>
+      </c>
+      <c r="K21" s="39">
         <f t="shared" si="0"/>
-        <v>0.47799422799422797</v>
-      </c>
-      <c r="L21" s="46">
+        <v>0.12964466089466087</v>
+      </c>
+      <c r="L21" s="44">
         <f t="shared" si="0"/>
-        <v>28.679653679653683</v>
-      </c>
-      <c r="M21" s="54">
+        <v>7.778679653679653</v>
+      </c>
+      <c r="M21" s="52">
         <f t="shared" si="0"/>
-        <v>229.43722943722946</v>
-      </c>
-      <c r="N21" s="47">
+        <v>62.229437229437224</v>
+      </c>
+      <c r="N21" s="45">
         <f t="shared" si="0"/>
-        <v>1104.1666666666667</v>
+        <v>299.47916666666674</v>
       </c>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="42">
+      <c r="B22" s="77"/>
+      <c r="C22" s="40">
         <f>C20-C18</f>
         <v>4.5281582952815839E-3</v>
       </c>
-      <c r="D22" s="48">
+      <c r="D22" s="46">
         <f t="shared" ref="D22:N22" si="1">D20-D18</f>
         <v>0.27168949771689499</v>
       </c>
-      <c r="E22" s="48">
+      <c r="E22" s="46">
         <f t="shared" si="1"/>
         <v>16.301369863013701</v>
       </c>
-      <c r="F22" s="48">
+      <c r="F22" s="46">
         <f t="shared" si="1"/>
         <v>391.23287671232879</v>
       </c>
-      <c r="G22" s="53">
+      <c r="G22" s="51">
         <f t="shared" si="1"/>
         <v>2746.1538461538462</v>
       </c>
-      <c r="H22" s="55">
+      <c r="H22" s="53">
         <f t="shared" si="1"/>
         <v>11900</v>
       </c>
-      <c r="I22" s="43">
+      <c r="I22" s="41">
         <f t="shared" si="1"/>
         <v>35700</v>
       </c>
-      <c r="J22" s="42">
+      <c r="J22" s="40">
         <f t="shared" si="1"/>
         <v>2.1464646464646468E-2</v>
       </c>
-      <c r="K22" s="53">
+      <c r="K22" s="51">
         <f t="shared" si="1"/>
         <v>1.2878787878787881</v>
       </c>
-      <c r="L22" s="53">
+      <c r="L22" s="51">
         <f t="shared" si="1"/>
         <v>77.27272727272728</v>
       </c>
-      <c r="M22" s="53">
+      <c r="M22" s="51">
         <f t="shared" si="1"/>
         <v>618.18181818181824</v>
       </c>
-      <c r="N22" s="43">
+      <c r="N22" s="41">
         <f t="shared" si="1"/>
         <v>3125</v>
       </c>
       <c r="O22" s="7"/>
     </row>
     <row r="23" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="44">
+      <c r="B23" s="75"/>
+      <c r="C23" s="42">
         <f>C20-C19</f>
-        <v>2.8475393201420605E-3</v>
-      </c>
-      <c r="D23" s="49">
+        <v>4.0723300355149684E-3</v>
+      </c>
+      <c r="D23" s="47">
         <f t="shared" ref="D23:N23" si="2">D20-D19</f>
-        <v>0.17085235920852362</v>
-      </c>
-      <c r="E23" s="49">
+        <v>0.24433980213089806</v>
+      </c>
+      <c r="E23" s="47">
         <f t="shared" si="2"/>
-        <v>10.251141552511417</v>
-      </c>
-      <c r="F23" s="51">
+        <v>14.660388127853881</v>
+      </c>
+      <c r="F23" s="49">
         <f t="shared" si="2"/>
-        <v>246.02739726027397</v>
-      </c>
-      <c r="G23" s="52">
+        <v>351.84931506849318</v>
+      </c>
+      <c r="G23" s="50">
         <f t="shared" si="2"/>
-        <v>1726.9230769230769</v>
-      </c>
-      <c r="H23" s="52">
+        <v>2469.7115384615381</v>
+      </c>
+      <c r="H23" s="50">
         <f t="shared" si="2"/>
-        <v>7483.333333333333</v>
-      </c>
-      <c r="I23" s="45">
+        <v>10702.083333333332</v>
+      </c>
+      <c r="I23" s="43">
         <f t="shared" si="2"/>
-        <v>22450</v>
-      </c>
-      <c r="J23" s="44">
+        <v>32106.25</v>
+      </c>
+      <c r="J23" s="42">
         <f t="shared" si="2"/>
-        <v>1.3498075998076E-2</v>
-      </c>
-      <c r="K23" s="52">
+        <v>1.9303902116402118E-2</v>
+      </c>
+      <c r="K23" s="50">
         <f t="shared" si="2"/>
-        <v>0.80988455988455998</v>
-      </c>
-      <c r="L23" s="52">
+        <v>1.158234126984127</v>
+      </c>
+      <c r="L23" s="50">
         <f t="shared" si="2"/>
-        <v>48.593073593073591</v>
-      </c>
-      <c r="M23" s="52">
+        <v>69.49404761904762</v>
+      </c>
+      <c r="M23" s="50">
         <f t="shared" si="2"/>
-        <v>388.74458874458873</v>
-      </c>
-      <c r="N23" s="45">
+        <v>555.95238095238096</v>
+      </c>
+      <c r="N23" s="43">
         <f t="shared" si="2"/>
-        <v>2020.8333333333333</v>
+        <v>2825.520833333333</v>
       </c>
       <c r="O23" s="7"/>
     </row>
     <row r="24" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="61"/>
-      <c r="E25" s="60">
+      <c r="D25" s="62"/>
+      <c r="E25" s="57">
         <f>100*(1-0.78299)</f>
         <v>21.701000000000004</v>
       </c>
-      <c r="F25" s="59"/>
+      <c r="F25" s="56"/>
     </row>
     <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -1619,351 +1644,360 @@
       </c>
     </row>
     <row r="29" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="61" t="s">
+      <c r="A29" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="62"/>
-      <c r="C29" s="16">
+      <c r="B29" s="77">
+        <f>$E$12</f>
+        <v>42000</v>
+      </c>
+      <c r="C29" s="15">
         <f>(((($E$12/365)/24)/60)/60) * (1 - ($E$25 / 100))</f>
         <v>1.0427949010654489E-3</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="16">
         <f>((($E$12/365)/24)/60) * (1 - ($E$25 / 100))</f>
         <v>6.256769406392694E-2</v>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="17">
         <f>(($E$12/365)/24) * (1 - ($E$25 / 100))</f>
         <v>3.754061643835616</v>
       </c>
-      <c r="F29" s="19">
+      <c r="F29" s="18">
         <f>($E$12/365) * (1 - ($E$25 / 100))</f>
         <v>90.097479452054785</v>
       </c>
-      <c r="G29" s="17">
+      <c r="G29" s="16">
         <f>($E$12/52) * (1 - ($E$25 / 100))</f>
         <v>632.41499999999996</v>
       </c>
-      <c r="H29" s="17">
+      <c r="H29" s="16">
         <f>($E$12/12) * (1 - ($E$25 / 100))</f>
         <v>2740.4649999999997</v>
       </c>
-      <c r="I29" s="20">
+      <c r="I29" s="19">
         <f>($E$12/4) * (1 - ($E$25 / 100))</f>
         <v>8221.3950000000004</v>
       </c>
-      <c r="J29" s="21">
+      <c r="J29" s="20">
         <f>$E$12/$F$6 * (1 - ($E$25 / 100))</f>
         <v>4.9431186868686867E-3</v>
       </c>
-      <c r="K29" s="22">
+      <c r="K29" s="21">
         <f>$E$12/$F$7 * (1 - ($E$25 / 100))</f>
         <v>0.29658712121212122</v>
       </c>
-      <c r="L29" s="19">
+      <c r="L29" s="18">
         <f>$E$12/$F$8 * (1 - ($E$25 / 100))</f>
         <v>17.795227272727271</v>
       </c>
-      <c r="M29" s="22">
+      <c r="M29" s="21">
         <f>$E$12/$F$3 * (1 - ($E$25 / 100))</f>
         <v>142.36181818181817</v>
       </c>
-      <c r="N29" s="23">
+      <c r="N29" s="22">
         <f>$E$12/$F$2 * (1 - ($E$25 / 100))</f>
         <v>685.11624999999992</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="62"/>
-      <c r="C30" s="24">
+      <c r="B30" s="75">
+        <f>$E$13</f>
+        <v>56375</v>
+      </c>
+      <c r="C30" s="23">
         <f>(((($E$13/365)/24)/60)/60) * (1 - ($E$25 / 100))</f>
-        <v>2.3587027524099441E-3</v>
-      </c>
-      <c r="D30" s="25">
+        <v>1.3997038701801115E-3</v>
+      </c>
+      <c r="D30" s="24">
         <f>((($E$13/365)/24)/60) * (1 - ($E$25 / 100))</f>
-        <v>0.14152216514459665</v>
-      </c>
-      <c r="E30" s="26">
+        <v>8.3982232210806682E-2</v>
+      </c>
+      <c r="E30" s="25">
         <f>(($E$13/365)/24) * (1 - ($E$25 / 100))</f>
-        <v>8.4913299086757981</v>
-      </c>
-      <c r="F30" s="27">
+        <v>5.0389339326484013</v>
+      </c>
+      <c r="F30" s="26">
         <f>($E$13/365) * (1 - ($E$25 / 100))</f>
-        <v>203.79191780821915</v>
-      </c>
-      <c r="G30" s="25">
+        <v>120.93441438356163</v>
+      </c>
+      <c r="G30" s="24">
         <f>($E$13/52) * (1 - ($E$25 / 100))</f>
-        <v>1430.4624999999999</v>
-      </c>
-      <c r="H30" s="25">
+        <v>848.86656249999999</v>
+      </c>
+      <c r="H30" s="24">
         <f>($E$13/12) * (1 - ($E$25 / 100))</f>
-        <v>6198.6708333333336</v>
-      </c>
-      <c r="I30" s="28">
+        <v>3678.4217708333335</v>
+      </c>
+      <c r="I30" s="27">
         <f>($E$13/4) * (1 - ($E$25 / 100))</f>
-        <v>18596.012500000001</v>
-      </c>
-      <c r="J30" s="29">
+        <v>11035.2653125</v>
+      </c>
+      <c r="J30" s="28">
         <f>$E$13/$F$6 * (1 - ($E$25 / 100))</f>
-        <v>1.1180863696488696E-2</v>
-      </c>
-      <c r="K30" s="30">
+        <v>6.634959904100529E-3</v>
+      </c>
+      <c r="K30" s="29">
         <f>$E$13/$F$7 * (1 - ($E$25 / 100))</f>
-        <v>0.67085182178932179</v>
-      </c>
-      <c r="L30" s="27">
+        <v>0.39809759424603169</v>
+      </c>
+      <c r="L30" s="26">
         <f>$E$13/$F$8 * (1 - ($E$25 / 100))</f>
-        <v>40.251109307359307</v>
-      </c>
-      <c r="M30" s="30">
+        <v>23.885855654761901</v>
+      </c>
+      <c r="M30" s="29">
         <f>$E$13/$F$3 * (1 - ($E$25 / 100))</f>
-        <v>322.00887445887446</v>
-      </c>
-      <c r="N30" s="31">
+        <v>191.08684523809521</v>
+      </c>
+      <c r="N30" s="30">
         <f>$E$13/$F$2 * (1 - ($E$25 / 100))</f>
-        <v>1549.6677083333334</v>
+        <v>919.60544270833338</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="32">
+      <c r="B31" s="79">
+        <f>$E$14</f>
+        <v>100</v>
+      </c>
+      <c r="C31" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60) * (1 - ($E$25 / 100))</f>
         <v>4.5882975646879759E-3</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="32">
         <f>$G$14/365 / 24 / 60 * (1 - ($E$25 / 100))</f>
         <v>0.27529785388127853</v>
       </c>
-      <c r="E31" s="33">
+      <c r="E31" s="32">
         <f>$G$14/365/24 * (1 - ($E$25 / 100))</f>
         <v>16.517871232876711</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="33">
         <f>$G$14 / 365 * (1 - ($E$25 / 100))</f>
         <v>396.4289095890411</v>
       </c>
-      <c r="G31" s="33">
+      <c r="G31" s="32">
         <f>$G$14 / 52 * (1 - ($E$25 / 100))</f>
         <v>2782.6259999999997</v>
       </c>
-      <c r="H31" s="33">
+      <c r="H31" s="32">
         <f>$G$14/12 * (1 - ($E$25 / 100))</f>
         <v>12058.046</v>
       </c>
-      <c r="I31" s="35">
+      <c r="I31" s="34">
         <f>$G$14/4 * (1 - ($E$25 / 100))</f>
         <v>36174.137999999999</v>
       </c>
-      <c r="J31" s="36">
+      <c r="J31" s="35">
         <f>(($E$14 / 60) / 60) * (1 - ($E$25 / 100))</f>
         <v>2.1749722222222222E-2</v>
       </c>
-      <c r="K31" s="34">
+      <c r="K31" s="33">
         <f>$E$14/60 * (1 - ($E$25 / 100))</f>
         <v>1.3049833333333334</v>
       </c>
-      <c r="L31" s="37">
+      <c r="L31" s="36">
         <f>$E$14 * (1 - ($E$25 / 100))</f>
         <v>78.298999999999992</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="37">
         <f>$E$14*$F$1 * (1 - ($E$25 / 100))</f>
         <v>626.39199999999994</v>
       </c>
-      <c r="N31" s="34">
+      <c r="N31" s="33">
         <f>$E$14*$F$1*5 * (1 - ($E$25 / 100))</f>
         <v>3131.96</v>
       </c>
       <c r="O31" s="7"/>
     </row>
     <row r="32" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="61" t="s">
+      <c r="A32" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="62"/>
-      <c r="C32" s="39">
+      <c r="B32" s="77"/>
+      <c r="C32" s="38">
         <f>C30-C29</f>
-        <v>1.3159078513444952E-3</v>
-      </c>
-      <c r="D32" s="46">
+        <v>3.5690896911466262E-4</v>
+      </c>
+      <c r="D32" s="44">
         <f t="shared" ref="D32:N32" si="3">D30-D29</f>
-        <v>7.8954471080669705E-2</v>
-      </c>
-      <c r="E32" s="50">
+        <v>2.1414538146879741E-2</v>
+      </c>
+      <c r="E32" s="48">
         <f t="shared" si="3"/>
-        <v>4.737268264840182</v>
-      </c>
-      <c r="F32" s="50">
+        <v>1.2848722888127853</v>
+      </c>
+      <c r="F32" s="48">
         <f t="shared" si="3"/>
-        <v>113.69443835616437</v>
-      </c>
-      <c r="G32" s="54">
+        <v>30.836934931506846</v>
+      </c>
+      <c r="G32" s="52">
         <f t="shared" si="3"/>
-        <v>798.0474999999999</v>
-      </c>
-      <c r="H32" s="46">
+        <v>216.45156250000002</v>
+      </c>
+      <c r="H32" s="44">
         <f t="shared" si="3"/>
-        <v>3458.2058333333339</v>
-      </c>
-      <c r="I32" s="47">
+        <v>937.95677083333385</v>
+      </c>
+      <c r="I32" s="45">
         <f t="shared" si="3"/>
-        <v>10374.6175</v>
-      </c>
-      <c r="J32" s="39">
+        <v>2813.8703124999993</v>
+      </c>
+      <c r="J32" s="38">
         <f t="shared" si="3"/>
-        <v>6.2377450096200091E-3</v>
-      </c>
-      <c r="K32" s="41">
+        <v>1.6918412172318422E-3</v>
+      </c>
+      <c r="K32" s="39">
         <f t="shared" si="3"/>
-        <v>0.37426470057720057</v>
-      </c>
-      <c r="L32" s="46">
+        <v>0.10151047303391048</v>
+      </c>
+      <c r="L32" s="44">
         <f t="shared" si="3"/>
-        <v>22.455882034632037</v>
-      </c>
-      <c r="M32" s="54">
+        <v>6.0906283820346303</v>
+      </c>
+      <c r="M32" s="52">
         <f t="shared" si="3"/>
-        <v>179.64705627705629</v>
-      </c>
-      <c r="N32" s="47">
+        <v>48.725027056277042</v>
+      </c>
+      <c r="N32" s="45">
         <f t="shared" si="3"/>
-        <v>864.55145833333347</v>
+        <v>234.48919270833346</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="61" t="s">
+      <c r="A33" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="62"/>
-      <c r="C33" s="42">
+      <c r="B33" s="77"/>
+      <c r="C33" s="40">
         <f>C31-C29</f>
         <v>3.545502663622527E-3</v>
       </c>
-      <c r="D33" s="48">
+      <c r="D33" s="46">
         <f t="shared" ref="D33:N33" si="4">D31-D29</f>
         <v>0.21273015981735161</v>
       </c>
-      <c r="E33" s="48">
+      <c r="E33" s="46">
         <f t="shared" si="4"/>
         <v>12.763809589041095</v>
       </c>
-      <c r="F33" s="48">
+      <c r="F33" s="46">
         <f t="shared" si="4"/>
         <v>306.33143013698634</v>
       </c>
-      <c r="G33" s="53">
+      <c r="G33" s="51">
         <f t="shared" si="4"/>
         <v>2150.2109999999998</v>
       </c>
-      <c r="H33" s="55">
+      <c r="H33" s="53">
         <f t="shared" si="4"/>
         <v>9317.5810000000001</v>
       </c>
-      <c r="I33" s="43">
+      <c r="I33" s="41">
         <f t="shared" si="4"/>
         <v>27952.742999999999</v>
       </c>
-      <c r="J33" s="42">
+      <c r="J33" s="40">
         <f t="shared" si="4"/>
         <v>1.6806603535353536E-2</v>
       </c>
-      <c r="K33" s="53">
+      <c r="K33" s="51">
         <f t="shared" si="4"/>
         <v>1.0083962121212122</v>
       </c>
-      <c r="L33" s="53">
+      <c r="L33" s="51">
         <f t="shared" si="4"/>
         <v>60.503772727272718</v>
       </c>
-      <c r="M33" s="53">
+      <c r="M33" s="51">
         <f t="shared" si="4"/>
         <v>484.03018181818175</v>
       </c>
-      <c r="N33" s="43">
+      <c r="N33" s="41">
         <f t="shared" si="4"/>
         <v>2446.84375</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="61" t="s">
+      <c r="A34" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="62"/>
-      <c r="C34" s="44">
+      <c r="B34" s="75"/>
+      <c r="C34" s="42">
         <f>C31-C30</f>
-        <v>2.2295948122780318E-3</v>
-      </c>
-      <c r="D34" s="49">
+        <v>3.1885936945078644E-3</v>
+      </c>
+      <c r="D34" s="47">
         <f t="shared" ref="D34:N34" si="5">D31-D30</f>
-        <v>0.13377568873668189</v>
-      </c>
-      <c r="E34" s="49">
+        <v>0.19131562167047184</v>
+      </c>
+      <c r="E34" s="47">
         <f t="shared" si="5"/>
-        <v>8.0265413242009132</v>
-      </c>
-      <c r="F34" s="51">
+        <v>11.47893730022831</v>
+      </c>
+      <c r="F34" s="49">
         <f t="shared" si="5"/>
-        <v>192.63699178082194</v>
-      </c>
-      <c r="G34" s="52">
+        <v>275.49449520547944</v>
+      </c>
+      <c r="G34" s="50">
         <f t="shared" si="5"/>
-        <v>1352.1634999999999</v>
-      </c>
-      <c r="H34" s="52">
+        <v>1933.7594374999999</v>
+      </c>
+      <c r="H34" s="50">
         <f t="shared" si="5"/>
-        <v>5859.3751666666667</v>
-      </c>
-      <c r="I34" s="45">
+        <v>8379.6242291666676</v>
+      </c>
+      <c r="I34" s="43">
         <f t="shared" si="5"/>
-        <v>17578.125499999998</v>
-      </c>
-      <c r="J34" s="44">
+        <v>25138.872687499999</v>
+      </c>
+      <c r="J34" s="42">
         <f t="shared" si="5"/>
-        <v>1.0568858525733527E-2</v>
-      </c>
-      <c r="K34" s="52">
+        <v>1.5114762318121693E-2</v>
+      </c>
+      <c r="K34" s="50">
         <f t="shared" si="5"/>
-        <v>0.63413151154401159</v>
-      </c>
-      <c r="L34" s="52">
+        <v>0.90688573908730175</v>
+      </c>
+      <c r="L34" s="50">
         <f t="shared" si="5"/>
-        <v>38.047890692640685</v>
-      </c>
-      <c r="M34" s="52">
+        <v>54.413144345238095</v>
+      </c>
+      <c r="M34" s="50">
         <f t="shared" si="5"/>
-        <v>304.38312554112548</v>
-      </c>
-      <c r="N34" s="45">
+        <v>435.30515476190476</v>
+      </c>
+      <c r="N34" s="43">
         <f t="shared" si="5"/>
-        <v>1582.2922916666666</v>
+        <v>2212.3545572916664</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
-      <c r="D37" s="67" t="s">
+      <c r="D37" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="67"/>
-      <c r="F37" s="67"/>
-      <c r="G37" s="67"/>
-      <c r="H37" s="67"/>
-      <c r="I37" s="67"/>
-      <c r="J37" s="70"/>
-      <c r="K37" s="69" t="s">
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="58"/>
+      <c r="J37" s="59"/>
+      <c r="K37" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="L37" s="67"/>
-      <c r="M37" s="67"/>
-      <c r="N37" s="67"/>
-      <c r="O37" s="67"/>
-      <c r="P37" s="67"/>
-      <c r="Q37" s="67"/>
+      <c r="L37" s="58"/>
+      <c r="M37" s="58"/>
+      <c r="N37" s="58"/>
+      <c r="O37" s="58"/>
+      <c r="P37" s="58"/>
+      <c r="Q37" s="58"/>
     </row>
     <row r="38" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C38" s="3" t="s">
@@ -3282,7 +3316,15 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="17">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="J16:N16"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="D37:J37"/>
     <mergeCell ref="K37:Q37"/>
     <mergeCell ref="C5:D5"/>
@@ -3292,19 +3334,6 @@
     <mergeCell ref="C27:I27"/>
     <mergeCell ref="J27:N27"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="J16:N16"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
2021-05-14 End of day file push
</commit_message>
<xml_diff>
--- a/Tax/calcs.xlsx
+++ b/Tax/calcs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABriggs\Documents\BWS\Tax\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD5F9C2-3090-4D77-8CDC-56D98DCCA050}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68F6A22-0798-4A24-8529-9AB51DE8E708}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3945" yWindow="1065" windowWidth="21600" windowHeight="11385" xr2:uid="{6D0CD4EE-CC56-4F74-B7F8-52D61ECC5DE1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6D0CD4EE-CC56-4F74-B7F8-52D61ECC5DE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -604,52 +604,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -668,6 +623,51 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1014,30 +1014,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="58"/>
+      <c r="D1" s="65"/>
       <c r="E1" s="66"/>
       <c r="F1" s="55">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="58"/>
+      <c r="D2" s="65"/>
       <c r="E2" s="66"/>
       <c r="F2" s="55">
         <v>48</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="58"/>
+      <c r="D3" s="65"/>
       <c r="E3" s="66"/>
       <c r="F3" s="54">
         <v>231</v>
@@ -1048,39 +1048,39 @@
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="61"/>
+      <c r="D5" s="78"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C6" s="61" t="s">
+      <c r="C6" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
+      <c r="D6" s="78"/>
+      <c r="E6" s="78"/>
       <c r="F6">
         <f>($F$3) * F1 * 60 * 60</f>
         <v>6652800</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
+      <c r="D7" s="78"/>
+      <c r="E7" s="78"/>
       <c r="F7">
         <f>($F$3) * F1 * 60</f>
         <v>110880</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C8" s="61" t="s">
+      <c r="C8" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
+      <c r="D8" s="78"/>
+      <c r="E8" s="78"/>
       <c r="F8">
         <f>($F$3) * F1</f>
         <v>1848</v>
@@ -1095,10 +1095,10 @@
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="69"/>
+      <c r="D12" s="75"/>
       <c r="E12" s="55">
         <v>42000</v>
       </c>
@@ -1117,19 +1117,19 @@
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C13" s="70" t="s">
+      <c r="C13" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="71"/>
+      <c r="D13" s="73"/>
       <c r="E13" s="54">
-        <v>56375</v>
+        <v>43000</v>
       </c>
       <c r="F13" t="s">
         <v>20</v>
       </c>
       <c r="G13">
         <f>E13</f>
-        <v>56375</v>
+        <v>43000</v>
       </c>
       <c r="H13" t="s">
         <v>20</v>
@@ -1140,19 +1140,19 @@
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
-      <c r="C14" s="72" t="s">
+      <c r="C14" s="76" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="73"/>
+      <c r="D14" s="77"/>
       <c r="E14" s="54">
-        <v>100</v>
+        <v>11.75</v>
       </c>
       <c r="F14" t="s">
         <v>21</v>
       </c>
       <c r="G14">
         <f>($E$14 * $F$1*$F$3)</f>
-        <v>184800</v>
+        <v>21714</v>
       </c>
       <c r="H14" t="s">
         <v>20</v>
@@ -1176,22 +1176,22 @@
       <c r="N15" s="4"/>
     </row>
     <row r="16" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="60" t="s">
+      <c r="C16" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
-      <c r="F16" s="58"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="63" t="s">
+      <c r="D16" s="65"/>
+      <c r="E16" s="65"/>
+      <c r="F16" s="65"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
+      <c r="I16" s="68"/>
+      <c r="J16" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="64"/>
-      <c r="L16" s="64"/>
-      <c r="M16" s="64"/>
-      <c r="N16" s="65"/>
+      <c r="K16" s="70"/>
+      <c r="L16" s="70"/>
+      <c r="M16" s="70"/>
+      <c r="N16" s="71"/>
       <c r="O16" s="13"/>
       <c r="P16" s="5"/>
     </row>
@@ -1236,10 +1236,10 @@
       <c r="P17" s="6"/>
     </row>
     <row r="18" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="76" t="s">
+      <c r="A18" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="77">
+      <c r="B18" s="62">
         <f>$E$12</f>
         <v>42000</v>
       </c>
@@ -1294,292 +1294,292 @@
       <c r="O18" s="7"/>
     </row>
     <row r="19" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="74" t="s">
+      <c r="A19" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="75">
+      <c r="B19" s="60">
         <f>$E$13</f>
-        <v>56375</v>
+        <v>43000</v>
       </c>
       <c r="C19" s="23">
         <f>(((($E$13/365)/24)/60)/60)</f>
-        <v>1.7876395230847285E-3</v>
+        <v>1.3635210553018774E-3</v>
       </c>
       <c r="D19" s="24">
         <f>((($E$13/365)/24)/60)</f>
-        <v>0.10725837138508371</v>
+        <v>8.1811263318112643E-2</v>
       </c>
       <c r="E19" s="25">
         <f>(($E$13/365)/24)</f>
-        <v>6.4355022831050226</v>
+        <v>4.9086757990867582</v>
       </c>
       <c r="F19" s="26">
         <f>($E$13/365)</f>
-        <v>154.45205479452054</v>
+        <v>117.8082191780822</v>
       </c>
       <c r="G19" s="24">
         <f>($E$13/52)</f>
-        <v>1084.1346153846155</v>
+        <v>826.92307692307691</v>
       </c>
       <c r="H19" s="24">
         <f>($E$13/12)</f>
-        <v>4697.916666666667</v>
+        <v>3583.3333333333335</v>
       </c>
       <c r="I19" s="27">
         <f>($E$13/4)</f>
-        <v>14093.75</v>
+        <v>10750</v>
       </c>
       <c r="J19" s="28">
         <f>$E$13/$F$6</f>
-        <v>8.4738756613756613E-3</v>
+        <v>6.4634439634439636E-3</v>
       </c>
       <c r="K19" s="29">
         <f>$E$13/$F$7</f>
-        <v>0.50843253968253965</v>
+        <v>0.38780663780663782</v>
       </c>
       <c r="L19" s="26">
         <f>$E$13/$F$8</f>
-        <v>30.50595238095238</v>
+        <v>23.268398268398268</v>
       </c>
       <c r="M19" s="29">
         <f>$E$13/$F$3</f>
-        <v>244.04761904761904</v>
+        <v>186.14718614718615</v>
       </c>
       <c r="N19" s="30">
         <f>$E$13/$F$2</f>
-        <v>1174.4791666666667</v>
+        <v>895.83333333333337</v>
       </c>
       <c r="O19" s="7"/>
     </row>
     <row r="20" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="78" t="s">
+      <c r="A20" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="79">
+      <c r="B20" s="64">
         <f>$E$14</f>
-        <v>100</v>
+        <v>11.75</v>
       </c>
       <c r="C20" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60)</f>
-        <v>5.8599695585996965E-3</v>
+        <v>6.8854642313546423E-4</v>
       </c>
       <c r="D20" s="32">
         <f>$G$14/365 / 24 / 60</f>
-        <v>0.35159817351598177</v>
+        <v>4.1312785388127854E-2</v>
       </c>
       <c r="E20" s="32">
         <f>$G$14/365/24</f>
-        <v>21.095890410958905</v>
+        <v>2.4787671232876711</v>
       </c>
       <c r="F20" s="33">
         <f>$G$14 / 365</f>
-        <v>506.30136986301369</v>
+        <v>59.490410958904107</v>
       </c>
       <c r="G20" s="32">
         <f>$G$14 / 52</f>
-        <v>3553.8461538461538</v>
+        <v>417.57692307692309</v>
       </c>
       <c r="H20" s="32">
         <f>$G$14/12</f>
-        <v>15400</v>
+        <v>1809.5</v>
       </c>
       <c r="I20" s="34">
         <f>$G$14/4</f>
-        <v>46200</v>
+        <v>5428.5</v>
       </c>
       <c r="J20" s="35">
         <f>(($E$14 / 60) / 60)</f>
-        <v>2.777777777777778E-2</v>
+        <v>3.2638888888888887E-3</v>
       </c>
       <c r="K20" s="33">
         <f>$E$14/60</f>
-        <v>1.6666666666666667</v>
+        <v>0.19583333333333333</v>
       </c>
       <c r="L20" s="36">
         <f>$E$14</f>
-        <v>100</v>
+        <v>11.75</v>
       </c>
       <c r="M20" s="37">
         <f>$E$14*$F$1</f>
-        <v>800</v>
+        <v>94</v>
       </c>
       <c r="N20" s="33">
         <f>$E$14*$F$1*5</f>
-        <v>4000</v>
+        <v>470</v>
       </c>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="74" t="s">
+      <c r="A21" s="59" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="77"/>
+      <c r="B21" s="62"/>
       <c r="C21" s="38">
         <f>C19-C18</f>
-        <v>4.5582825976661591E-4</v>
+        <v>3.1709791983764802E-5</v>
       </c>
       <c r="D21" s="44">
         <f t="shared" ref="D21:N21" si="0">D19-D18</f>
-        <v>2.7349695585996953E-2</v>
+        <v>1.902587519025889E-3</v>
       </c>
       <c r="E21" s="48">
         <f t="shared" si="0"/>
-        <v>1.6409817351598175</v>
+        <v>0.11415525114155312</v>
       </c>
       <c r="F21" s="48">
         <f t="shared" si="0"/>
-        <v>39.383561643835606</v>
+        <v>2.7397260273972677</v>
       </c>
       <c r="G21" s="52">
         <f t="shared" si="0"/>
-        <v>276.44230769230774</v>
+        <v>19.23076923076917</v>
       </c>
       <c r="H21" s="44">
         <f>H19-H18</f>
-        <v>1197.916666666667</v>
+        <v>83.333333333333485</v>
       </c>
       <c r="I21" s="45">
         <f t="shared" si="0"/>
-        <v>3593.75</v>
+        <v>250</v>
       </c>
       <c r="J21" s="38">
         <f t="shared" si="0"/>
-        <v>2.1607443482443483E-3</v>
+        <v>1.5031265031265062E-4</v>
       </c>
       <c r="K21" s="39">
         <f t="shared" si="0"/>
-        <v>0.12964466089466087</v>
+        <v>9.0187590187590372E-3</v>
       </c>
       <c r="L21" s="44">
         <f t="shared" si="0"/>
-        <v>7.778679653679653</v>
+        <v>0.54112554112554179</v>
       </c>
       <c r="M21" s="52">
         <f t="shared" si="0"/>
-        <v>62.229437229437224</v>
+        <v>4.3290043290043343</v>
       </c>
       <c r="N21" s="45">
         <f t="shared" si="0"/>
-        <v>299.47916666666674</v>
+        <v>20.833333333333371</v>
       </c>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="77"/>
+      <c r="B22" s="62"/>
       <c r="C22" s="40">
         <f>C20-C18</f>
-        <v>4.5281582952815839E-3</v>
+        <v>-6.4326484018264833E-4</v>
       </c>
       <c r="D22" s="46">
         <f t="shared" ref="D22:N22" si="1">D20-D18</f>
-        <v>0.27168949771689499</v>
+        <v>-3.85958904109589E-2</v>
       </c>
       <c r="E22" s="46">
         <f t="shared" si="1"/>
-        <v>16.301369863013701</v>
+        <v>-2.315753424657534</v>
       </c>
       <c r="F22" s="46">
         <f t="shared" si="1"/>
-        <v>391.23287671232879</v>
+        <v>-55.578082191780823</v>
       </c>
       <c r="G22" s="51">
         <f t="shared" si="1"/>
-        <v>2746.1538461538462</v>
+        <v>-390.11538461538464</v>
       </c>
       <c r="H22" s="53">
         <f t="shared" si="1"/>
-        <v>11900</v>
+        <v>-1690.5</v>
       </c>
       <c r="I22" s="41">
         <f t="shared" si="1"/>
-        <v>35700</v>
+        <v>-5071.5</v>
       </c>
       <c r="J22" s="40">
         <f t="shared" si="1"/>
-        <v>2.1464646464646468E-2</v>
+        <v>-3.0492424242424244E-3</v>
       </c>
       <c r="K22" s="51">
         <f t="shared" si="1"/>
-        <v>1.2878787878787881</v>
+        <v>-0.18295454545454545</v>
       </c>
       <c r="L22" s="51">
         <f t="shared" si="1"/>
-        <v>77.27272727272728</v>
+        <v>-10.977272727272727</v>
       </c>
       <c r="M22" s="51">
         <f t="shared" si="1"/>
-        <v>618.18181818181824</v>
+        <v>-87.818181818181813</v>
       </c>
       <c r="N22" s="41">
         <f t="shared" si="1"/>
-        <v>3125</v>
+        <v>-405</v>
       </c>
       <c r="O22" s="7"/>
     </row>
     <row r="23" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="75"/>
+      <c r="B23" s="60"/>
       <c r="C23" s="42">
         <f>C20-C19</f>
-        <v>4.0723300355149684E-3</v>
+        <v>-6.7497463216641314E-4</v>
       </c>
       <c r="D23" s="47">
         <f t="shared" ref="D23:N23" si="2">D20-D19</f>
-        <v>0.24433980213089806</v>
+        <v>-4.0498477929984789E-2</v>
       </c>
       <c r="E23" s="47">
         <f t="shared" si="2"/>
-        <v>14.660388127853881</v>
+        <v>-2.4299086757990871</v>
       </c>
       <c r="F23" s="49">
         <f t="shared" si="2"/>
-        <v>351.84931506849318</v>
+        <v>-58.31780821917809</v>
       </c>
       <c r="G23" s="50">
         <f t="shared" si="2"/>
-        <v>2469.7115384615381</v>
+        <v>-409.34615384615381</v>
       </c>
       <c r="H23" s="50">
         <f t="shared" si="2"/>
-        <v>10702.083333333332</v>
+        <v>-1773.8333333333335</v>
       </c>
       <c r="I23" s="43">
         <f t="shared" si="2"/>
-        <v>32106.25</v>
+        <v>-5321.5</v>
       </c>
       <c r="J23" s="42">
         <f t="shared" si="2"/>
-        <v>1.9303902116402118E-2</v>
+        <v>-3.199555074555075E-3</v>
       </c>
       <c r="K23" s="50">
         <f t="shared" si="2"/>
-        <v>1.158234126984127</v>
+        <v>-0.19197330447330449</v>
       </c>
       <c r="L23" s="50">
         <f t="shared" si="2"/>
-        <v>69.49404761904762</v>
+        <v>-11.518398268398268</v>
       </c>
       <c r="M23" s="50">
         <f t="shared" si="2"/>
-        <v>555.95238095238096</v>
+        <v>-92.147186147186147</v>
       </c>
       <c r="N23" s="43">
         <f t="shared" si="2"/>
-        <v>2825.520833333333</v>
+        <v>-425.83333333333337</v>
       </c>
       <c r="O23" s="7"/>
     </row>
     <row r="24" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C25" s="62" t="s">
+      <c r="C25" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="62"/>
+      <c r="D25" s="79"/>
       <c r="E25" s="57">
         <f>100*(1-0.78299)</f>
         <v>21.701000000000004</v>
@@ -1588,22 +1588,22 @@
     </row>
     <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="63" t="s">
+      <c r="C27" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="64"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="65"/>
-      <c r="J27" s="63" t="s">
+      <c r="D27" s="70"/>
+      <c r="E27" s="70"/>
+      <c r="F27" s="70"/>
+      <c r="G27" s="70"/>
+      <c r="H27" s="70"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="K27" s="64"/>
-      <c r="L27" s="64"/>
-      <c r="M27" s="64"/>
-      <c r="N27" s="65"/>
+      <c r="K27" s="70"/>
+      <c r="L27" s="70"/>
+      <c r="M27" s="70"/>
+      <c r="N27" s="71"/>
     </row>
     <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="10" t="s">
@@ -1644,10 +1644,10 @@
       </c>
     </row>
     <row r="29" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="76" t="s">
+      <c r="A29" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="77">
+      <c r="B29" s="62">
         <f>$E$12</f>
         <v>42000</v>
       </c>
@@ -1701,303 +1701,303 @@
       </c>
     </row>
     <row r="30" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="74" t="s">
+      <c r="A30" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="75">
+      <c r="B30" s="60">
         <f>$E$13</f>
-        <v>56375</v>
+        <v>43000</v>
       </c>
       <c r="C30" s="23">
         <f>(((($E$13/365)/24)/60)/60) * (1 - ($E$25 / 100))</f>
-        <v>1.3997038701801115E-3</v>
+        <v>1.067623351090817E-3</v>
       </c>
       <c r="D30" s="24">
         <f>((($E$13/365)/24)/60) * (1 - ($E$25 / 100))</f>
-        <v>8.3982232210806682E-2</v>
+        <v>6.4057401065449021E-2</v>
       </c>
       <c r="E30" s="25">
         <f>(($E$13/365)/24) * (1 - ($E$25 / 100))</f>
-        <v>5.0389339326484013</v>
+        <v>3.8434440639269405</v>
       </c>
       <c r="F30" s="26">
         <f>($E$13/365) * (1 - ($E$25 / 100))</f>
-        <v>120.93441438356163</v>
+        <v>92.242657534246575</v>
       </c>
       <c r="G30" s="24">
         <f>($E$13/52) * (1 - ($E$25 / 100))</f>
-        <v>848.86656249999999</v>
+        <v>647.47249999999997</v>
       </c>
       <c r="H30" s="24">
         <f>($E$13/12) * (1 - ($E$25 / 100))</f>
-        <v>3678.4217708333335</v>
+        <v>2805.7141666666666</v>
       </c>
       <c r="I30" s="27">
         <f>($E$13/4) * (1 - ($E$25 / 100))</f>
-        <v>11035.2653125</v>
+        <v>8417.1424999999999</v>
       </c>
       <c r="J30" s="28">
         <f>$E$13/$F$6 * (1 - ($E$25 / 100))</f>
-        <v>6.634959904100529E-3</v>
+        <v>5.0608119889369889E-3</v>
       </c>
       <c r="K30" s="29">
         <f>$E$13/$F$7 * (1 - ($E$25 / 100))</f>
-        <v>0.39809759424603169</v>
+        <v>0.30364871933621934</v>
       </c>
       <c r="L30" s="26">
         <f>$E$13/$F$8 * (1 - ($E$25 / 100))</f>
-        <v>23.885855654761901</v>
+        <v>18.218923160173158</v>
       </c>
       <c r="M30" s="29">
         <f>$E$13/$F$3 * (1 - ($E$25 / 100))</f>
-        <v>191.08684523809521</v>
+        <v>145.75138528138527</v>
       </c>
       <c r="N30" s="30">
         <f>$E$13/$F$2 * (1 - ($E$25 / 100))</f>
-        <v>919.60544270833338</v>
+        <v>701.42854166666666</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="78" t="s">
+      <c r="A31" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="79">
+      <c r="B31" s="64">
         <f>$E$14</f>
-        <v>100</v>
+        <v>11.75</v>
       </c>
       <c r="C31" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60) * (1 - ($E$25 / 100))</f>
-        <v>4.5882975646879759E-3</v>
+        <v>5.3912496385083713E-4</v>
       </c>
       <c r="D31" s="32">
         <f>$G$14/365 / 24 / 60 * (1 - ($E$25 / 100))</f>
-        <v>0.27529785388127853</v>
+        <v>3.2347497831050225E-2</v>
       </c>
       <c r="E31" s="32">
         <f>$G$14/365/24 * (1 - ($E$25 / 100))</f>
-        <v>16.517871232876711</v>
+        <v>1.9408498698630134</v>
       </c>
       <c r="F31" s="33">
         <f>$G$14 / 365 * (1 - ($E$25 / 100))</f>
-        <v>396.4289095890411</v>
+        <v>46.580396876712328</v>
       </c>
       <c r="G31" s="32">
         <f>$G$14 / 52 * (1 - ($E$25 / 100))</f>
-        <v>2782.6259999999997</v>
+        <v>326.95855499999999</v>
       </c>
       <c r="H31" s="32">
         <f>$G$14/12 * (1 - ($E$25 / 100))</f>
-        <v>12058.046</v>
+        <v>1416.8204049999999</v>
       </c>
       <c r="I31" s="34">
         <f>$G$14/4 * (1 - ($E$25 / 100))</f>
-        <v>36174.137999999999</v>
+        <v>4250.4612149999994</v>
       </c>
       <c r="J31" s="35">
         <f>(($E$14 / 60) / 60) * (1 - ($E$25 / 100))</f>
-        <v>2.1749722222222222E-2</v>
+        <v>2.5555923611111108E-3</v>
       </c>
       <c r="K31" s="33">
         <f>$E$14/60 * (1 - ($E$25 / 100))</f>
-        <v>1.3049833333333334</v>
+        <v>0.15333554166666666</v>
       </c>
       <c r="L31" s="36">
         <f>$E$14 * (1 - ($E$25 / 100))</f>
-        <v>78.298999999999992</v>
+        <v>9.2001324999999987</v>
       </c>
       <c r="M31" s="37">
         <f>$E$14*$F$1 * (1 - ($E$25 / 100))</f>
-        <v>626.39199999999994</v>
+        <v>73.60105999999999</v>
       </c>
       <c r="N31" s="33">
         <f>$E$14*$F$1*5 * (1 - ($E$25 / 100))</f>
-        <v>3131.96</v>
+        <v>368.00529999999998</v>
       </c>
       <c r="O31" s="7"/>
     </row>
     <row r="32" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="74" t="s">
+      <c r="A32" s="59" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="77"/>
+      <c r="B32" s="62"/>
       <c r="C32" s="38">
         <f>C30-C29</f>
-        <v>3.5690896911466262E-4</v>
+        <v>2.4828450025368059E-5</v>
       </c>
       <c r="D32" s="44">
         <f t="shared" ref="D32:N32" si="3">D30-D29</f>
-        <v>2.1414538146879741E-2</v>
+        <v>1.4897070015220809E-3</v>
       </c>
       <c r="E32" s="48">
         <f t="shared" si="3"/>
-        <v>1.2848722888127853</v>
+        <v>8.9382420091324466E-2</v>
       </c>
       <c r="F32" s="48">
         <f t="shared" si="3"/>
-        <v>30.836934931506846</v>
+        <v>2.1451780821917907</v>
       </c>
       <c r="G32" s="52">
         <f t="shared" si="3"/>
-        <v>216.45156250000002</v>
+        <v>15.057500000000005</v>
       </c>
       <c r="H32" s="44">
         <f t="shared" si="3"/>
-        <v>937.95677083333385</v>
+        <v>65.249166666666952</v>
       </c>
       <c r="I32" s="45">
         <f t="shared" si="3"/>
-        <v>2813.8703124999993</v>
+        <v>195.74749999999949</v>
       </c>
       <c r="J32" s="38">
         <f t="shared" si="3"/>
-        <v>1.6918412172318422E-3</v>
+        <v>1.1769330206830211E-4</v>
       </c>
       <c r="K32" s="39">
         <f t="shared" si="3"/>
-        <v>0.10151047303391048</v>
+        <v>7.0615981240981229E-3</v>
       </c>
       <c r="L32" s="44">
         <f t="shared" si="3"/>
-        <v>6.0906283820346303</v>
+        <v>0.42369588744588782</v>
       </c>
       <c r="M32" s="52">
         <f t="shared" si="3"/>
-        <v>48.725027056277042</v>
+        <v>3.3895670995671026</v>
       </c>
       <c r="N32" s="45">
         <f t="shared" si="3"/>
-        <v>234.48919270833346</v>
+        <v>16.312291666666738</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="67" t="s">
+      <c r="A33" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="77"/>
+      <c r="B33" s="62"/>
       <c r="C33" s="40">
         <f>C31-C29</f>
-        <v>3.545502663622527E-3</v>
+        <v>-5.0366993721461179E-4</v>
       </c>
       <c r="D33" s="46">
         <f t="shared" ref="D33:N33" si="4">D31-D29</f>
-        <v>0.21273015981735161</v>
+        <v>-3.0220196232876716E-2</v>
       </c>
       <c r="E33" s="46">
         <f t="shared" si="4"/>
-        <v>12.763809589041095</v>
+        <v>-1.8132117739726026</v>
       </c>
       <c r="F33" s="46">
         <f t="shared" si="4"/>
-        <v>306.33143013698634</v>
+        <v>-43.517082575342457</v>
       </c>
       <c r="G33" s="51">
         <f t="shared" si="4"/>
-        <v>2150.2109999999998</v>
+        <v>-305.45644499999997</v>
       </c>
       <c r="H33" s="53">
         <f t="shared" si="4"/>
-        <v>9317.5810000000001</v>
+        <v>-1323.6445949999998</v>
       </c>
       <c r="I33" s="41">
         <f t="shared" si="4"/>
-        <v>27952.742999999999</v>
+        <v>-3970.9337850000011</v>
       </c>
       <c r="J33" s="40">
         <f t="shared" si="4"/>
-        <v>1.6806603535353536E-2</v>
+        <v>-2.3875263257575759E-3</v>
       </c>
       <c r="K33" s="51">
         <f t="shared" si="4"/>
-        <v>1.0083962121212122</v>
+        <v>-0.14325157954545456</v>
       </c>
       <c r="L33" s="51">
         <f t="shared" si="4"/>
-        <v>60.503772727272718</v>
+        <v>-8.595094772727272</v>
       </c>
       <c r="M33" s="51">
         <f t="shared" si="4"/>
-        <v>484.03018181818175</v>
+        <v>-68.760758181818176</v>
       </c>
       <c r="N33" s="41">
         <f t="shared" si="4"/>
-        <v>2446.84375</v>
+        <v>-317.11094999999995</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="67" t="s">
+      <c r="A34" s="58" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="75"/>
+      <c r="B34" s="60"/>
       <c r="C34" s="42">
         <f>C31-C30</f>
-        <v>3.1885936945078644E-3</v>
+        <v>-5.2849838723997985E-4</v>
       </c>
       <c r="D34" s="47">
         <f t="shared" ref="D34:N34" si="5">D31-D30</f>
-        <v>0.19131562167047184</v>
+        <v>-3.1709903234398797E-2</v>
       </c>
       <c r="E34" s="47">
         <f t="shared" si="5"/>
-        <v>11.47893730022831</v>
+        <v>-1.902594194063927</v>
       </c>
       <c r="F34" s="49">
         <f t="shared" si="5"/>
-        <v>275.49449520547944</v>
+        <v>-45.662260657534247</v>
       </c>
       <c r="G34" s="50">
         <f t="shared" si="5"/>
-        <v>1933.7594374999999</v>
+        <v>-320.51394499999998</v>
       </c>
       <c r="H34" s="50">
         <f t="shared" si="5"/>
-        <v>8379.6242291666676</v>
+        <v>-1388.8937616666667</v>
       </c>
       <c r="I34" s="43">
         <f t="shared" si="5"/>
-        <v>25138.872687499999</v>
+        <v>-4166.6812850000006</v>
       </c>
       <c r="J34" s="42">
         <f t="shared" si="5"/>
-        <v>1.5114762318121693E-2</v>
+        <v>-2.505219627825878E-3</v>
       </c>
       <c r="K34" s="50">
         <f t="shared" si="5"/>
-        <v>0.90688573908730175</v>
+        <v>-0.15031317766955268</v>
       </c>
       <c r="L34" s="50">
         <f t="shared" si="5"/>
-        <v>54.413144345238095</v>
+        <v>-9.0187906601731598</v>
       </c>
       <c r="M34" s="50">
         <f t="shared" si="5"/>
-        <v>435.30515476190476</v>
+        <v>-72.150325281385278</v>
       </c>
       <c r="N34" s="43">
         <f t="shared" si="5"/>
-        <v>2212.3545572916664</v>
+        <v>-333.42324166666668</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
-      <c r="D37" s="58" t="s">
+      <c r="D37" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
-      <c r="G37" s="58"/>
-      <c r="H37" s="58"/>
-      <c r="I37" s="58"/>
-      <c r="J37" s="59"/>
-      <c r="K37" s="60" t="s">
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="68"/>
+      <c r="K37" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="L37" s="58"/>
-      <c r="M37" s="58"/>
-      <c r="N37" s="58"/>
-      <c r="O37" s="58"/>
-      <c r="P37" s="58"/>
-      <c r="Q37" s="58"/>
+      <c r="L37" s="65"/>
+      <c r="M37" s="65"/>
+      <c r="N37" s="65"/>
+      <c r="O37" s="65"/>
+      <c r="P37" s="65"/>
+      <c r="Q37" s="65"/>
     </row>
     <row r="38" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C38" s="3" t="s">
@@ -3317,14 +3317,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="J16:N16"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C14:D14"/>
     <mergeCell ref="D37:J37"/>
     <mergeCell ref="K37:Q37"/>
     <mergeCell ref="C5:D5"/>
@@ -3334,6 +3326,14 @@
     <mergeCell ref="C27:I27"/>
     <mergeCell ref="J27:N27"/>
     <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="J16:N16"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
2021-05-19 End of day file push
</commit_message>
<xml_diff>
--- a/Tax/calcs.xlsx
+++ b/Tax/calcs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABriggs\Documents\BWS\Tax\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68F6A22-0798-4A24-8529-9AB51DE8E708}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F227577D-2429-4135-AD53-B8B5924A7E3A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6D0CD4EE-CC56-4F74-B7F8-52D61ECC5DE1}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6D0CD4EE-CC56-4F74-B7F8-52D61ECC5DE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -628,14 +628,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -644,6 +647,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -662,12 +668,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1018,7 +1018,7 @@
         <v>7</v>
       </c>
       <c r="D1" s="65"/>
-      <c r="E1" s="66"/>
+      <c r="E1" s="73"/>
       <c r="F1" s="55">
         <v>8</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>14</v>
       </c>
       <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
+      <c r="E2" s="73"/>
       <c r="F2" s="55">
         <v>48</v>
       </c>
@@ -1038,9 +1038,9 @@
         <v>8</v>
       </c>
       <c r="D3" s="65"/>
-      <c r="E3" s="66"/>
+      <c r="E3" s="73"/>
       <c r="F3" s="54">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.25">
@@ -1048,42 +1048,42 @@
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C5" s="78" t="s">
+      <c r="C5" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="78"/>
+      <c r="D5" s="68"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C6" s="78" t="s">
+      <c r="C6" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
       <c r="F6">
         <f>($F$3) * F1 * 60 * 60</f>
-        <v>6652800</v>
+        <v>6940800</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C7" s="78" t="s">
+      <c r="C7" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
       <c r="F7">
         <f>($F$3) * F1 * 60</f>
-        <v>110880</v>
+        <v>115680</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C8" s="78" t="s">
+      <c r="C8" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="78"/>
-      <c r="E8" s="78"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
       <c r="F8">
         <f>($F$3) * F1</f>
-        <v>1848</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
@@ -1095,10 +1095,10 @@
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C12" s="74" t="s">
+      <c r="C12" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="75"/>
+      <c r="D12" s="77"/>
       <c r="E12" s="55">
         <v>42000</v>
       </c>
@@ -1117,19 +1117,19 @@
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="74" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="73"/>
+      <c r="D13" s="75"/>
       <c r="E13" s="54">
-        <v>43000</v>
+        <v>63000</v>
       </c>
       <c r="F13" t="s">
         <v>20</v>
       </c>
       <c r="G13">
         <f>E13</f>
-        <v>43000</v>
+        <v>63000</v>
       </c>
       <c r="H13" t="s">
         <v>20</v>
@@ -1140,19 +1140,19 @@
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
-      <c r="C14" s="76" t="s">
+      <c r="C14" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="77"/>
+      <c r="D14" s="79"/>
       <c r="E14" s="54">
-        <v>11.75</v>
+        <v>36.54</v>
       </c>
       <c r="F14" t="s">
         <v>21</v>
       </c>
       <c r="G14">
         <f>($E$14 * $F$1*$F$3)</f>
-        <v>21714</v>
+        <v>70449.119999999995</v>
       </c>
       <c r="H14" t="s">
         <v>20</v>
@@ -1184,14 +1184,14 @@
       <c r="F16" s="65"/>
       <c r="G16" s="65"/>
       <c r="H16" s="65"/>
-      <c r="I16" s="68"/>
-      <c r="J16" s="69" t="s">
+      <c r="I16" s="66"/>
+      <c r="J16" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="70"/>
-      <c r="L16" s="70"/>
-      <c r="M16" s="70"/>
-      <c r="N16" s="71"/>
+      <c r="K16" s="71"/>
+      <c r="L16" s="71"/>
+      <c r="M16" s="71"/>
+      <c r="N16" s="72"/>
       <c r="O16" s="13"/>
       <c r="P16" s="5"/>
     </row>
@@ -1273,19 +1273,19 @@
       </c>
       <c r="J18" s="20">
         <f>$E$12/$F$6</f>
-        <v>6.313131313131313E-3</v>
+        <v>6.0511756569847858E-3</v>
       </c>
       <c r="K18" s="21">
         <f>$E$12/$F$7</f>
-        <v>0.37878787878787878</v>
+        <v>0.36307053941908712</v>
       </c>
       <c r="L18" s="18">
         <f>$E$12/$F$8</f>
-        <v>22.727272727272727</v>
+        <v>21.784232365145229</v>
       </c>
       <c r="M18" s="21">
         <f>$E$12/$F$3</f>
-        <v>181.81818181818181</v>
+        <v>174.27385892116183</v>
       </c>
       <c r="N18" s="22">
         <f>$E$12/$F$2</f>
@@ -1299,55 +1299,55 @@
       </c>
       <c r="B19" s="60">
         <f>$E$13</f>
-        <v>43000</v>
+        <v>63000</v>
       </c>
       <c r="C19" s="23">
         <f>(((($E$13/365)/24)/60)/60)</f>
-        <v>1.3635210553018774E-3</v>
+        <v>1.9977168949771693E-3</v>
       </c>
       <c r="D19" s="24">
         <f>((($E$13/365)/24)/60)</f>
-        <v>8.1811263318112643E-2</v>
+        <v>0.11986301369863014</v>
       </c>
       <c r="E19" s="25">
         <f>(($E$13/365)/24)</f>
-        <v>4.9086757990867582</v>
+        <v>7.191780821917809</v>
       </c>
       <c r="F19" s="26">
         <f>($E$13/365)</f>
-        <v>117.8082191780822</v>
+        <v>172.60273972602741</v>
       </c>
       <c r="G19" s="24">
         <f>($E$13/52)</f>
-        <v>826.92307692307691</v>
+        <v>1211.5384615384614</v>
       </c>
       <c r="H19" s="24">
         <f>($E$13/12)</f>
-        <v>3583.3333333333335</v>
+        <v>5250</v>
       </c>
       <c r="I19" s="27">
         <f>($E$13/4)</f>
-        <v>10750</v>
+        <v>15750</v>
       </c>
       <c r="J19" s="28">
         <f>$E$13/$F$6</f>
-        <v>6.4634439634439636E-3</v>
+        <v>9.0767634854771791E-3</v>
       </c>
       <c r="K19" s="29">
         <f>$E$13/$F$7</f>
-        <v>0.38780663780663782</v>
+        <v>0.54460580912863066</v>
       </c>
       <c r="L19" s="26">
         <f>$E$13/$F$8</f>
-        <v>23.268398268398268</v>
+        <v>32.676348547717843</v>
       </c>
       <c r="M19" s="29">
         <f>$E$13/$F$3</f>
-        <v>186.14718614718615</v>
+        <v>261.41078838174275</v>
       </c>
       <c r="N19" s="30">
         <f>$E$13/$F$2</f>
-        <v>895.83333333333337</v>
+        <v>1312.5</v>
       </c>
       <c r="O19" s="7"/>
     </row>
@@ -1357,55 +1357,55 @@
       </c>
       <c r="B20" s="64">
         <f>$E$14</f>
-        <v>11.75</v>
+        <v>36.54</v>
       </c>
       <c r="C20" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60)</f>
-        <v>6.8854642313546423E-4</v>
+        <v>2.2339269406392694E-3</v>
       </c>
       <c r="D20" s="32">
         <f>$G$14/365 / 24 / 60</f>
-        <v>4.1312785388127854E-2</v>
+        <v>0.13403561643835615</v>
       </c>
       <c r="E20" s="32">
         <f>$G$14/365/24</f>
-        <v>2.4787671232876711</v>
+        <v>8.0421369863013688</v>
       </c>
       <c r="F20" s="33">
         <f>$G$14 / 365</f>
-        <v>59.490410958904107</v>
+        <v>193.01128767123285</v>
       </c>
       <c r="G20" s="32">
         <f>$G$14 / 52</f>
-        <v>417.57692307692309</v>
+        <v>1354.7907692307692</v>
       </c>
       <c r="H20" s="32">
         <f>$G$14/12</f>
-        <v>1809.5</v>
+        <v>5870.7599999999993</v>
       </c>
       <c r="I20" s="34">
         <f>$G$14/4</f>
-        <v>5428.5</v>
+        <v>17612.28</v>
       </c>
       <c r="J20" s="35">
         <f>(($E$14 / 60) / 60)</f>
-        <v>3.2638888888888887E-3</v>
+        <v>1.0149999999999999E-2</v>
       </c>
       <c r="K20" s="33">
         <f>$E$14/60</f>
-        <v>0.19583333333333333</v>
+        <v>0.60899999999999999</v>
       </c>
       <c r="L20" s="36">
         <f>$E$14</f>
-        <v>11.75</v>
+        <v>36.54</v>
       </c>
       <c r="M20" s="37">
         <f>$E$14*$F$1</f>
-        <v>94</v>
+        <v>292.32</v>
       </c>
       <c r="N20" s="33">
         <f>$E$14*$F$1*5</f>
-        <v>470</v>
+        <v>1461.6</v>
       </c>
       <c r="O20" s="7"/>
     </row>
@@ -1416,51 +1416,51 @@
       <c r="B21" s="62"/>
       <c r="C21" s="38">
         <f>C19-C18</f>
-        <v>3.1709791983764802E-5</v>
+        <v>6.6590563165905671E-4</v>
       </c>
       <c r="D21" s="44">
         <f t="shared" ref="D21:N21" si="0">D19-D18</f>
-        <v>1.902587519025889E-3</v>
+        <v>3.9954337899543391E-2</v>
       </c>
       <c r="E21" s="48">
         <f t="shared" si="0"/>
-        <v>0.11415525114155312</v>
+        <v>2.3972602739726039</v>
       </c>
       <c r="F21" s="48">
         <f t="shared" si="0"/>
-        <v>2.7397260273972677</v>
+        <v>57.534246575342479</v>
       </c>
       <c r="G21" s="52">
         <f t="shared" si="0"/>
-        <v>19.23076923076917</v>
+        <v>403.8461538461537</v>
       </c>
       <c r="H21" s="44">
         <f>H19-H18</f>
-        <v>83.333333333333485</v>
+        <v>1750</v>
       </c>
       <c r="I21" s="45">
         <f t="shared" si="0"/>
-        <v>250</v>
+        <v>5250</v>
       </c>
       <c r="J21" s="38">
         <f t="shared" si="0"/>
-        <v>1.5031265031265062E-4</v>
+        <v>3.0255878284923933E-3</v>
       </c>
       <c r="K21" s="39">
         <f t="shared" si="0"/>
-        <v>9.0187590187590372E-3</v>
+        <v>0.18153526970954353</v>
       </c>
       <c r="L21" s="44">
         <f t="shared" si="0"/>
-        <v>0.54112554112554179</v>
+        <v>10.892116182572614</v>
       </c>
       <c r="M21" s="52">
         <f t="shared" si="0"/>
-        <v>4.3290043290043343</v>
+        <v>87.136929460580916</v>
       </c>
       <c r="N21" s="45">
         <f t="shared" si="0"/>
-        <v>20.833333333333371</v>
+        <v>437.5</v>
       </c>
       <c r="O21" s="7"/>
     </row>
@@ -1471,51 +1471,51 @@
       <c r="B22" s="62"/>
       <c r="C22" s="40">
         <f>C20-C18</f>
-        <v>-6.4326484018264833E-4</v>
+        <v>9.0211567732115683E-4</v>
       </c>
       <c r="D22" s="46">
         <f t="shared" ref="D22:N22" si="1">D20-D18</f>
-        <v>-3.85958904109589E-2</v>
+        <v>5.41269406392694E-2</v>
       </c>
       <c r="E22" s="46">
         <f t="shared" si="1"/>
-        <v>-2.315753424657534</v>
+        <v>3.2476164383561636</v>
       </c>
       <c r="F22" s="46">
         <f t="shared" si="1"/>
-        <v>-55.578082191780823</v>
+        <v>77.94279452054792</v>
       </c>
       <c r="G22" s="51">
         <f t="shared" si="1"/>
-        <v>-390.11538461538464</v>
+        <v>547.09846153846149</v>
       </c>
       <c r="H22" s="53">
         <f t="shared" si="1"/>
-        <v>-1690.5</v>
+        <v>2370.7599999999993</v>
       </c>
       <c r="I22" s="41">
         <f t="shared" si="1"/>
-        <v>-5071.5</v>
+        <v>7112.2799999999988</v>
       </c>
       <c r="J22" s="40">
         <f t="shared" si="1"/>
-        <v>-3.0492424242424244E-3</v>
+        <v>4.0988243430152135E-3</v>
       </c>
       <c r="K22" s="51">
         <f t="shared" si="1"/>
-        <v>-0.18295454545454545</v>
+        <v>0.24592946058091286</v>
       </c>
       <c r="L22" s="51">
         <f t="shared" si="1"/>
-        <v>-10.977272727272727</v>
+        <v>14.75576763485477</v>
       </c>
       <c r="M22" s="51">
         <f t="shared" si="1"/>
-        <v>-87.818181818181813</v>
+        <v>118.04614107883816</v>
       </c>
       <c r="N22" s="41">
         <f t="shared" si="1"/>
-        <v>-405</v>
+        <v>586.59999999999991</v>
       </c>
       <c r="O22" s="7"/>
     </row>
@@ -1526,60 +1526,60 @@
       <c r="B23" s="60"/>
       <c r="C23" s="42">
         <f>C20-C19</f>
-        <v>-6.7497463216641314E-4</v>
+        <v>2.3621004566210012E-4</v>
       </c>
       <c r="D23" s="47">
         <f t="shared" ref="D23:N23" si="2">D20-D19</f>
-        <v>-4.0498477929984789E-2</v>
+        <v>1.4172602739726009E-2</v>
       </c>
       <c r="E23" s="47">
         <f t="shared" si="2"/>
-        <v>-2.4299086757990871</v>
+        <v>0.85035616438355976</v>
       </c>
       <c r="F23" s="49">
         <f t="shared" si="2"/>
-        <v>-58.31780821917809</v>
+        <v>20.408547945205441</v>
       </c>
       <c r="G23" s="50">
         <f t="shared" si="2"/>
-        <v>-409.34615384615381</v>
+        <v>143.2523076923078</v>
       </c>
       <c r="H23" s="50">
         <f t="shared" si="2"/>
-        <v>-1773.8333333333335</v>
+        <v>620.75999999999931</v>
       </c>
       <c r="I23" s="43">
         <f t="shared" si="2"/>
-        <v>-5321.5</v>
+        <v>1862.2799999999988</v>
       </c>
       <c r="J23" s="42">
         <f t="shared" si="2"/>
-        <v>-3.199555074555075E-3</v>
+        <v>1.0732365145228202E-3</v>
       </c>
       <c r="K23" s="50">
         <f t="shared" si="2"/>
-        <v>-0.19197330447330449</v>
+        <v>6.4394190871369328E-2</v>
       </c>
       <c r="L23" s="50">
         <f t="shared" si="2"/>
-        <v>-11.518398268398268</v>
+        <v>3.8636514522821557</v>
       </c>
       <c r="M23" s="50">
         <f t="shared" si="2"/>
-        <v>-92.147186147186147</v>
+        <v>30.909211618257245</v>
       </c>
       <c r="N23" s="43">
         <f t="shared" si="2"/>
-        <v>-425.83333333333337</v>
+        <v>149.09999999999991</v>
       </c>
       <c r="O23" s="7"/>
     </row>
     <row r="24" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C25" s="79" t="s">
+      <c r="C25" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="79"/>
+      <c r="D25" s="69"/>
       <c r="E25" s="57">
         <f>100*(1-0.78299)</f>
         <v>21.701000000000004</v>
@@ -1588,22 +1588,22 @@
     </row>
     <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="69" t="s">
+      <c r="C27" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="70"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="71"/>
-      <c r="J27" s="69" t="s">
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="72"/>
+      <c r="J27" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="K27" s="70"/>
-      <c r="L27" s="70"/>
-      <c r="M27" s="70"/>
-      <c r="N27" s="71"/>
+      <c r="K27" s="71"/>
+      <c r="L27" s="71"/>
+      <c r="M27" s="71"/>
+      <c r="N27" s="72"/>
     </row>
     <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="10" t="s">
@@ -1681,19 +1681,19 @@
       </c>
       <c r="J29" s="20">
         <f>$E$12/$F$6 * (1 - ($E$25 / 100))</f>
-        <v>4.9431186868686867E-3</v>
+        <v>4.7380100276625172E-3</v>
       </c>
       <c r="K29" s="21">
         <f>$E$12/$F$7 * (1 - ($E$25 / 100))</f>
-        <v>0.29658712121212122</v>
+        <v>0.284280601659751</v>
       </c>
       <c r="L29" s="18">
         <f>$E$12/$F$8 * (1 - ($E$25 / 100))</f>
-        <v>17.795227272727271</v>
+        <v>17.056836099585063</v>
       </c>
       <c r="M29" s="21">
         <f>$E$12/$F$3 * (1 - ($E$25 / 100))</f>
-        <v>142.36181818181817</v>
+        <v>136.4546887966805</v>
       </c>
       <c r="N29" s="22">
         <f>$E$12/$F$2 * (1 - ($E$25 / 100))</f>
@@ -1706,55 +1706,55 @@
       </c>
       <c r="B30" s="60">
         <f>$E$13</f>
-        <v>43000</v>
+        <v>63000</v>
       </c>
       <c r="C30" s="23">
         <f>(((($E$13/365)/24)/60)/60) * (1 - ($E$25 / 100))</f>
-        <v>1.067623351090817E-3</v>
+        <v>1.5641923515981736E-3</v>
       </c>
       <c r="D30" s="24">
         <f>((($E$13/365)/24)/60) * (1 - ($E$25 / 100))</f>
-        <v>6.4057401065449021E-2</v>
+        <v>9.3851541095890417E-2</v>
       </c>
       <c r="E30" s="25">
         <f>(($E$13/365)/24) * (1 - ($E$25 / 100))</f>
-        <v>3.8434440639269405</v>
+        <v>5.6310924657534249</v>
       </c>
       <c r="F30" s="26">
         <f>($E$13/365) * (1 - ($E$25 / 100))</f>
-        <v>92.242657534246575</v>
+        <v>135.14621917808219</v>
       </c>
       <c r="G30" s="24">
         <f>($E$13/52) * (1 - ($E$25 / 100))</f>
-        <v>647.47249999999997</v>
+        <v>948.62249999999983</v>
       </c>
       <c r="H30" s="24">
         <f>($E$13/12) * (1 - ($E$25 / 100))</f>
-        <v>2805.7141666666666</v>
+        <v>4110.6975000000002</v>
       </c>
       <c r="I30" s="27">
         <f>($E$13/4) * (1 - ($E$25 / 100))</f>
-        <v>8417.1424999999999</v>
+        <v>12332.092499999999</v>
       </c>
       <c r="J30" s="28">
         <f>$E$13/$F$6 * (1 - ($E$25 / 100))</f>
-        <v>5.0608119889369889E-3</v>
+        <v>7.1070150414937758E-3</v>
       </c>
       <c r="K30" s="29">
         <f>$E$13/$F$7 * (1 - ($E$25 / 100))</f>
-        <v>0.30364871933621934</v>
+        <v>0.4264209024896265</v>
       </c>
       <c r="L30" s="26">
         <f>$E$13/$F$8 * (1 - ($E$25 / 100))</f>
-        <v>18.218923160173158</v>
+        <v>25.585254149377594</v>
       </c>
       <c r="M30" s="29">
         <f>$E$13/$F$3 * (1 - ($E$25 / 100))</f>
-        <v>145.75138528138527</v>
+        <v>204.68203319502075</v>
       </c>
       <c r="N30" s="30">
         <f>$E$13/$F$2 * (1 - ($E$25 / 100))</f>
-        <v>701.42854166666666</v>
+        <v>1027.6743750000001</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1763,55 +1763,55 @@
       </c>
       <c r="B31" s="64">
         <f>$E$14</f>
-        <v>11.75</v>
+        <v>36.54</v>
       </c>
       <c r="C31" s="31">
         <f>(((($G$14 / 365) / 24) / 60) / 60) * (1 - ($E$25 / 100))</f>
-        <v>5.3912496385083713E-4</v>
+        <v>1.7491424552511414E-3</v>
       </c>
       <c r="D31" s="32">
         <f>$G$14/365 / 24 / 60 * (1 - ($E$25 / 100))</f>
-        <v>3.2347497831050225E-2</v>
+        <v>0.10494854731506847</v>
       </c>
       <c r="E31" s="32">
         <f>$G$14/365/24 * (1 - ($E$25 / 100))</f>
-        <v>1.9408498698630134</v>
+        <v>6.2969128389041087</v>
       </c>
       <c r="F31" s="33">
         <f>$G$14 / 365 * (1 - ($E$25 / 100))</f>
-        <v>46.580396876712328</v>
+        <v>151.1259081336986</v>
       </c>
       <c r="G31" s="32">
         <f>$G$14 / 52 * (1 - ($E$25 / 100))</f>
-        <v>326.95855499999999</v>
+        <v>1060.7876243999999</v>
       </c>
       <c r="H31" s="32">
         <f>$G$14/12 * (1 - ($E$25 / 100))</f>
-        <v>1416.8204049999999</v>
+        <v>4596.746372399999</v>
       </c>
       <c r="I31" s="34">
         <f>$G$14/4 * (1 - ($E$25 / 100))</f>
-        <v>4250.4612149999994</v>
+        <v>13790.239117199999</v>
       </c>
       <c r="J31" s="35">
         <f>(($E$14 / 60) / 60) * (1 - ($E$25 / 100))</f>
-        <v>2.5555923611111108E-3</v>
+        <v>7.9473484999999996E-3</v>
       </c>
       <c r="K31" s="33">
         <f>$E$14/60 * (1 - ($E$25 / 100))</f>
-        <v>0.15333554166666666</v>
+        <v>0.47684090999999995</v>
       </c>
       <c r="L31" s="36">
         <f>$E$14 * (1 - ($E$25 / 100))</f>
-        <v>9.2001324999999987</v>
+        <v>28.610454599999997</v>
       </c>
       <c r="M31" s="37">
         <f>$E$14*$F$1 * (1 - ($E$25 / 100))</f>
-        <v>73.60105999999999</v>
+        <v>228.88363679999998</v>
       </c>
       <c r="N31" s="33">
         <f>$E$14*$F$1*5 * (1 - ($E$25 / 100))</f>
-        <v>368.00529999999998</v>
+        <v>1144.4181839999999</v>
       </c>
       <c r="O31" s="7"/>
     </row>
@@ -1822,51 +1822,51 @@
       <c r="B32" s="62"/>
       <c r="C32" s="38">
         <f>C30-C29</f>
-        <v>2.4828450025368059E-5</v>
+        <v>5.2139745053272468E-4</v>
       </c>
       <c r="D32" s="44">
         <f t="shared" ref="D32:N32" si="3">D30-D29</f>
-        <v>1.4897070015220809E-3</v>
+        <v>3.1283847031963477E-2</v>
       </c>
       <c r="E32" s="48">
         <f t="shared" si="3"/>
-        <v>8.9382420091324466E-2</v>
+        <v>1.8770308219178089</v>
       </c>
       <c r="F32" s="48">
         <f t="shared" si="3"/>
-        <v>2.1451780821917907</v>
+        <v>45.048739726027407</v>
       </c>
       <c r="G32" s="52">
         <f t="shared" si="3"/>
-        <v>15.057500000000005</v>
+        <v>316.20749999999987</v>
       </c>
       <c r="H32" s="44">
         <f t="shared" si="3"/>
-        <v>65.249166666666952</v>
+        <v>1370.2325000000005</v>
       </c>
       <c r="I32" s="45">
         <f t="shared" si="3"/>
-        <v>195.74749999999949</v>
+        <v>4110.6974999999984</v>
       </c>
       <c r="J32" s="38">
         <f t="shared" si="3"/>
-        <v>1.1769330206830211E-4</v>
+        <v>2.3690050138312586E-3</v>
       </c>
       <c r="K32" s="39">
         <f t="shared" si="3"/>
-        <v>7.0615981240981229E-3</v>
+        <v>0.1421403008298755</v>
       </c>
       <c r="L32" s="44">
         <f t="shared" si="3"/>
-        <v>0.42369588744588782</v>
+        <v>8.5284180497925313</v>
       </c>
       <c r="M32" s="52">
         <f t="shared" si="3"/>
-        <v>3.3895670995671026</v>
+        <v>68.22734439834025</v>
       </c>
       <c r="N32" s="45">
         <f t="shared" si="3"/>
-        <v>16.312291666666738</v>
+        <v>342.55812500000013</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1876,51 +1876,51 @@
       <c r="B33" s="62"/>
       <c r="C33" s="40">
         <f>C31-C29</f>
-        <v>-5.0366993721461179E-4</v>
+        <v>7.0634755418569253E-4</v>
       </c>
       <c r="D33" s="46">
         <f t="shared" ref="D33:N33" si="4">D31-D29</f>
-        <v>-3.0220196232876716E-2</v>
+        <v>4.2380853251141534E-2</v>
       </c>
       <c r="E33" s="46">
         <f t="shared" si="4"/>
-        <v>-1.8132117739726026</v>
+        <v>2.5428511950684927</v>
       </c>
       <c r="F33" s="46">
         <f t="shared" si="4"/>
-        <v>-43.517082575342457</v>
+        <v>61.028428681643817</v>
       </c>
       <c r="G33" s="51">
         <f t="shared" si="4"/>
-        <v>-305.45644499999997</v>
+        <v>428.37262439999995</v>
       </c>
       <c r="H33" s="53">
         <f t="shared" si="4"/>
-        <v>-1323.6445949999998</v>
+        <v>1856.2813723999993</v>
       </c>
       <c r="I33" s="41">
         <f t="shared" si="4"/>
-        <v>-3970.9337850000011</v>
+        <v>5568.8441171999984</v>
       </c>
       <c r="J33" s="40">
         <f t="shared" si="4"/>
-        <v>-2.3875263257575759E-3</v>
+        <v>3.2093384723374824E-3</v>
       </c>
       <c r="K33" s="51">
         <f t="shared" si="4"/>
-        <v>-0.14325157954545456</v>
+        <v>0.19256030834024895</v>
       </c>
       <c r="L33" s="51">
         <f t="shared" si="4"/>
-        <v>-8.595094772727272</v>
+        <v>11.553618500414935</v>
       </c>
       <c r="M33" s="51">
         <f t="shared" si="4"/>
-        <v>-68.760758181818176</v>
+        <v>92.428948003319476</v>
       </c>
       <c r="N33" s="41">
         <f t="shared" si="4"/>
-        <v>-317.11094999999995</v>
+        <v>459.30193399999996</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1930,51 +1930,51 @@
       <c r="B34" s="60"/>
       <c r="C34" s="42">
         <f>C31-C30</f>
-        <v>-5.2849838723997985E-4</v>
+        <v>1.8495010365296785E-4</v>
       </c>
       <c r="D34" s="47">
         <f t="shared" ref="D34:N34" si="5">D31-D30</f>
-        <v>-3.1709903234398797E-2</v>
+        <v>1.1097006219178057E-2</v>
       </c>
       <c r="E34" s="47">
         <f t="shared" si="5"/>
-        <v>-1.902594194063927</v>
+        <v>0.66582037315068376</v>
       </c>
       <c r="F34" s="49">
         <f t="shared" si="5"/>
-        <v>-45.662260657534247</v>
+        <v>15.97968895561641</v>
       </c>
       <c r="G34" s="50">
         <f t="shared" si="5"/>
-        <v>-320.51394499999998</v>
+        <v>112.16512440000008</v>
       </c>
       <c r="H34" s="50">
         <f t="shared" si="5"/>
-        <v>-1388.8937616666667</v>
+        <v>486.0488723999988</v>
       </c>
       <c r="I34" s="43">
         <f t="shared" si="5"/>
-        <v>-4166.6812850000006</v>
+        <v>1458.1466172</v>
       </c>
       <c r="J34" s="42">
         <f t="shared" si="5"/>
-        <v>-2.505219627825878E-3</v>
+        <v>8.4033345850622384E-4</v>
       </c>
       <c r="K34" s="50">
         <f t="shared" si="5"/>
-        <v>-0.15031317766955268</v>
+        <v>5.0420007510373455E-2</v>
       </c>
       <c r="L34" s="50">
         <f t="shared" si="5"/>
-        <v>-9.0187906601731598</v>
+        <v>3.0252004506224033</v>
       </c>
       <c r="M34" s="50">
         <f t="shared" si="5"/>
-        <v>-72.150325281385278</v>
+        <v>24.201603604979226</v>
       </c>
       <c r="N34" s="43">
         <f t="shared" si="5"/>
-        <v>-333.42324166666668</v>
+        <v>116.74380899999983</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -1988,7 +1988,7 @@
       <c r="G37" s="65"/>
       <c r="H37" s="65"/>
       <c r="I37" s="65"/>
-      <c r="J37" s="68"/>
+      <c r="J37" s="66"/>
       <c r="K37" s="67" t="s">
         <v>17</v>
       </c>
@@ -2076,19 +2076,19 @@
       </c>
       <c r="K39">
         <f>C39/$F$6</f>
-        <v>7.5156325156325161E-5</v>
+        <v>7.2037805440295068E-5</v>
       </c>
       <c r="L39">
         <f>C39 / $F$7</f>
-        <v>4.5093795093795091E-3</v>
+        <v>4.3222683264177043E-3</v>
       </c>
       <c r="M39">
         <f t="shared" ref="M39:M62" si="6">C39/$F$8</f>
-        <v>0.27056277056277056</v>
+        <v>0.25933609958506226</v>
       </c>
       <c r="N39">
         <f t="shared" ref="N39:N62" si="7">C39/$F$3</f>
-        <v>2.1645021645021645</v>
+        <v>2.0746887966804981</v>
       </c>
       <c r="O39">
         <f t="shared" ref="O39:O62" si="8">C39/$F$2</f>
@@ -2130,19 +2130,19 @@
       </c>
       <c r="K40">
         <f>C40/$F$6</f>
-        <v>1.5031265031265032E-4</v>
+        <v>1.4407561088059014E-4</v>
       </c>
       <c r="L40">
         <f t="shared" ref="L40:L62" si="16">C40 / $F$7</f>
-        <v>9.0187590187590181E-3</v>
+        <v>8.6445366528354085E-3</v>
       </c>
       <c r="M40">
         <f t="shared" si="6"/>
-        <v>0.54112554112554112</v>
+        <v>0.51867219917012453</v>
       </c>
       <c r="N40">
         <f t="shared" si="7"/>
-        <v>4.329004329004329</v>
+        <v>4.1493775933609962</v>
       </c>
       <c r="O40">
         <f t="shared" si="8"/>
@@ -2183,19 +2183,19 @@
       </c>
       <c r="K41">
         <f t="shared" ref="K41:K62" si="17">C41/$F$6</f>
-        <v>3.0062530062530064E-4</v>
+        <v>2.8815122176118027E-4</v>
       </c>
       <c r="L41">
         <f t="shared" si="16"/>
-        <v>1.8037518037518036E-2</v>
+        <v>1.7289073305670817E-2</v>
       </c>
       <c r="M41">
         <f t="shared" si="6"/>
-        <v>1.0822510822510822</v>
+        <v>1.0373443983402491</v>
       </c>
       <c r="N41">
         <f t="shared" si="7"/>
-        <v>8.6580086580086579</v>
+        <v>8.2987551867219924</v>
       </c>
       <c r="O41">
         <f t="shared" si="8"/>
@@ -2236,19 +2236,19 @@
       </c>
       <c r="K42">
         <f t="shared" si="17"/>
-        <v>3.7578162578162579E-4</v>
+        <v>3.6018902720147536E-4</v>
       </c>
       <c r="L42">
         <f t="shared" si="16"/>
-        <v>2.2546897546897548E-2</v>
+        <v>2.161134163208852E-2</v>
       </c>
       <c r="M42">
         <f t="shared" si="6"/>
-        <v>1.3528138528138529</v>
+        <v>1.2966804979253113</v>
       </c>
       <c r="N42">
         <f t="shared" si="7"/>
-        <v>10.822510822510823</v>
+        <v>10.37344398340249</v>
       </c>
       <c r="O42">
         <f t="shared" si="8"/>
@@ -2289,19 +2289,19 @@
       </c>
       <c r="K43">
         <f t="shared" si="17"/>
-        <v>7.5156325156325158E-4</v>
+        <v>7.2037805440295071E-4</v>
       </c>
       <c r="L43">
         <f t="shared" si="16"/>
-        <v>4.5093795093795096E-2</v>
+        <v>4.3222683264177039E-2</v>
       </c>
       <c r="M43">
         <f t="shared" si="6"/>
-        <v>2.7056277056277058</v>
+        <v>2.5933609958506225</v>
       </c>
       <c r="N43">
         <f t="shared" si="7"/>
-        <v>21.645021645021647</v>
+        <v>20.74688796680498</v>
       </c>
       <c r="O43">
         <f t="shared" si="8"/>
@@ -2342,19 +2342,19 @@
       </c>
       <c r="K44">
         <f t="shared" si="17"/>
-        <v>1.5031265031265032E-3</v>
+        <v>1.4407561088059014E-3</v>
       </c>
       <c r="L44">
         <f t="shared" si="16"/>
-        <v>9.0187590187590191E-2</v>
+        <v>8.6445366528354078E-2</v>
       </c>
       <c r="M44">
         <f t="shared" si="6"/>
-        <v>5.4112554112554117</v>
+        <v>5.186721991701245</v>
       </c>
       <c r="N44">
         <f t="shared" si="7"/>
-        <v>43.290043290043293</v>
+        <v>41.49377593360996</v>
       </c>
       <c r="O44">
         <f t="shared" si="8"/>
@@ -2395,19 +2395,19 @@
       </c>
       <c r="K45">
         <f t="shared" si="17"/>
-        <v>2.2546897546897545E-3</v>
+        <v>2.1611341632088521E-3</v>
       </c>
       <c r="L45">
         <f t="shared" si="16"/>
-        <v>0.13528138528138528</v>
+        <v>0.12966804979253113</v>
       </c>
       <c r="M45">
         <f t="shared" si="6"/>
-        <v>8.1168831168831161</v>
+        <v>7.7800829875518671</v>
       </c>
       <c r="N45">
         <f t="shared" si="7"/>
-        <v>64.935064935064929</v>
+        <v>62.240663900414937</v>
       </c>
       <c r="O45">
         <f t="shared" si="8"/>
@@ -2448,19 +2448,19 @@
       </c>
       <c r="K46">
         <f t="shared" si="17"/>
-        <v>3.0062530062530063E-3</v>
+        <v>2.8815122176118028E-3</v>
       </c>
       <c r="L46">
         <f t="shared" si="16"/>
-        <v>0.18037518037518038</v>
+        <v>0.17289073305670816</v>
       </c>
       <c r="M46">
         <f t="shared" si="6"/>
-        <v>10.822510822510823</v>
+        <v>10.37344398340249</v>
       </c>
       <c r="N46">
         <f t="shared" si="7"/>
-        <v>86.580086580086586</v>
+        <v>82.987551867219921</v>
       </c>
       <c r="O46">
         <f t="shared" si="8"/>
@@ -2501,19 +2501,19 @@
       </c>
       <c r="K47">
         <f t="shared" si="17"/>
-        <v>3.7578162578162577E-3</v>
+        <v>3.6018902720147536E-3</v>
       </c>
       <c r="L47">
         <f t="shared" si="16"/>
-        <v>0.22546897546897546</v>
+        <v>0.21611341632088521</v>
       </c>
       <c r="M47">
         <f t="shared" si="6"/>
-        <v>13.528138528138529</v>
+        <v>12.966804979253112</v>
       </c>
       <c r="N47">
         <f t="shared" si="7"/>
-        <v>108.22510822510823</v>
+        <v>103.7344398340249</v>
       </c>
       <c r="O47">
         <f t="shared" si="8"/>
@@ -2554,19 +2554,19 @@
       </c>
       <c r="K48">
         <f t="shared" si="17"/>
-        <v>4.5093795093795091E-3</v>
+        <v>4.3222683264177043E-3</v>
       </c>
       <c r="L48">
         <f t="shared" si="16"/>
-        <v>0.27056277056277056</v>
+        <v>0.25933609958506226</v>
       </c>
       <c r="M48">
         <f t="shared" si="6"/>
-        <v>16.233766233766232</v>
+        <v>15.560165975103734</v>
       </c>
       <c r="N48">
         <f t="shared" si="7"/>
-        <v>129.87012987012986</v>
+        <v>124.48132780082987</v>
       </c>
       <c r="O48">
         <f t="shared" si="8"/>
@@ -2607,19 +2607,19 @@
       </c>
       <c r="K49">
         <f t="shared" si="17"/>
-        <v>5.2609427609427613E-3</v>
+        <v>5.042646380820655E-3</v>
       </c>
       <c r="L49">
         <f t="shared" si="16"/>
-        <v>0.31565656565656564</v>
+        <v>0.30255878284923926</v>
       </c>
       <c r="M49">
         <f t="shared" si="6"/>
-        <v>18.939393939393938</v>
+        <v>18.153526970954356</v>
       </c>
       <c r="N49">
         <f t="shared" si="7"/>
-        <v>151.5151515151515</v>
+        <v>145.22821576763485</v>
       </c>
       <c r="O49">
         <f t="shared" si="8"/>
@@ -2660,19 +2660,19 @@
       </c>
       <c r="K50">
         <f t="shared" si="17"/>
-        <v>6.0125060125060126E-3</v>
+        <v>5.7630244352236057E-3</v>
       </c>
       <c r="L50">
         <f t="shared" si="16"/>
-        <v>0.36075036075036077</v>
+        <v>0.34578146611341631</v>
       </c>
       <c r="M50">
         <f t="shared" si="6"/>
-        <v>21.645021645021647</v>
+        <v>20.74688796680498</v>
       </c>
       <c r="N50">
         <f t="shared" si="7"/>
-        <v>173.16017316017317</v>
+        <v>165.97510373443984</v>
       </c>
       <c r="O50">
         <f t="shared" si="8"/>
@@ -2713,19 +2713,19 @@
       </c>
       <c r="K51">
         <f t="shared" si="17"/>
-        <v>6.764069264069264E-3</v>
+        <v>6.4834024896265564E-3</v>
       </c>
       <c r="L51">
         <f t="shared" si="16"/>
-        <v>0.40584415584415584</v>
+        <v>0.38900414937759337</v>
       </c>
       <c r="M51">
         <f t="shared" si="6"/>
-        <v>24.350649350649352</v>
+        <v>23.3402489626556</v>
       </c>
       <c r="N51">
         <f t="shared" si="7"/>
-        <v>194.80519480519482</v>
+        <v>186.7219917012448</v>
       </c>
       <c r="O51">
         <f t="shared" si="8"/>
@@ -2766,19 +2766,19 @@
       </c>
       <c r="K52">
         <f t="shared" si="17"/>
-        <v>7.5156325156325154E-3</v>
+        <v>7.2037805440295071E-3</v>
       </c>
       <c r="L52">
         <f t="shared" si="16"/>
-        <v>0.45093795093795092</v>
+        <v>0.43222683264177042</v>
       </c>
       <c r="M52">
         <f t="shared" si="6"/>
-        <v>27.056277056277057</v>
+        <v>25.933609958506224</v>
       </c>
       <c r="N52">
         <f t="shared" si="7"/>
-        <v>216.45021645021646</v>
+        <v>207.46887966804979</v>
       </c>
       <c r="O52">
         <f t="shared" si="8"/>
@@ -2819,19 +2819,19 @@
       </c>
       <c r="K53">
         <f t="shared" si="17"/>
-        <v>8.2671957671957667E-3</v>
+        <v>7.924158598432457E-3</v>
       </c>
       <c r="L53">
         <f t="shared" si="16"/>
-        <v>0.49603174603174605</v>
+        <v>0.47544951590594742</v>
       </c>
       <c r="M53">
         <f t="shared" si="6"/>
-        <v>29.761904761904763</v>
+        <v>28.526970954356848</v>
       </c>
       <c r="N53">
         <f t="shared" si="7"/>
-        <v>238.0952380952381</v>
+        <v>228.21576763485479</v>
       </c>
       <c r="O53">
         <f t="shared" si="8"/>
@@ -2872,19 +2872,19 @@
       </c>
       <c r="K54">
         <f t="shared" si="17"/>
-        <v>9.0187590187590181E-3</v>
+        <v>8.6445366528354085E-3</v>
       </c>
       <c r="L54">
         <f t="shared" si="16"/>
-        <v>0.54112554112554112</v>
+        <v>0.51867219917012453</v>
       </c>
       <c r="M54">
         <f t="shared" si="6"/>
-        <v>32.467532467532465</v>
+        <v>31.120331950207468</v>
       </c>
       <c r="N54">
         <f t="shared" si="7"/>
-        <v>259.74025974025972</v>
+        <v>248.96265560165975</v>
       </c>
       <c r="O54">
         <f t="shared" si="8"/>
@@ -2925,19 +2925,19 @@
       </c>
       <c r="K55">
         <f t="shared" si="17"/>
-        <v>9.7703222703222695E-3</v>
+        <v>9.3649147072383584E-3</v>
       </c>
       <c r="L55">
         <f t="shared" si="16"/>
-        <v>0.5862193362193362</v>
+        <v>0.56189488243430152</v>
       </c>
       <c r="M55">
         <f t="shared" si="6"/>
-        <v>35.17316017316017</v>
+        <v>33.713692946058089</v>
       </c>
       <c r="N55">
         <f t="shared" si="7"/>
-        <v>281.38528138528136</v>
+        <v>269.70954356846471</v>
       </c>
       <c r="O55">
         <f t="shared" si="8"/>
@@ -2978,19 +2978,19 @@
       </c>
       <c r="K56">
         <f t="shared" si="17"/>
-        <v>1.0521885521885523E-2</v>
+        <v>1.008529276164131E-2</v>
       </c>
       <c r="L56">
         <f t="shared" si="16"/>
-        <v>0.63131313131313127</v>
+        <v>0.60511756569847852</v>
       </c>
       <c r="M56">
         <f t="shared" si="6"/>
-        <v>37.878787878787875</v>
+        <v>36.307053941908713</v>
       </c>
       <c r="N56">
         <f t="shared" si="7"/>
-        <v>303.030303030303</v>
+        <v>290.4564315352697</v>
       </c>
       <c r="O56">
         <f t="shared" si="8"/>
@@ -3031,19 +3031,19 @@
       </c>
       <c r="K57">
         <f t="shared" si="17"/>
-        <v>1.1273448773448774E-2</v>
+        <v>1.080567081604426E-2</v>
       </c>
       <c r="L57">
         <f t="shared" si="16"/>
-        <v>0.67640692640692646</v>
+        <v>0.64834024896265563</v>
       </c>
       <c r="M57">
         <f t="shared" si="6"/>
-        <v>40.584415584415588</v>
+        <v>38.900414937759336</v>
       </c>
       <c r="N57">
         <f t="shared" si="7"/>
-        <v>324.6753246753247</v>
+        <v>311.20331950207469</v>
       </c>
       <c r="O57">
         <f t="shared" si="8"/>
@@ -3084,19 +3084,19 @@
       </c>
       <c r="K58">
         <f t="shared" si="17"/>
-        <v>1.2025012025012025E-2</v>
+        <v>1.1526048870447211E-2</v>
       </c>
       <c r="L58">
         <f t="shared" si="16"/>
-        <v>0.72150072150072153</v>
+        <v>0.69156293222683263</v>
       </c>
       <c r="M58">
         <f t="shared" si="6"/>
-        <v>43.290043290043293</v>
+        <v>41.49377593360996</v>
       </c>
       <c r="N58">
         <f t="shared" si="7"/>
-        <v>346.32034632034635</v>
+        <v>331.95020746887968</v>
       </c>
       <c r="O58">
         <f t="shared" si="8"/>
@@ -3137,19 +3137,19 @@
       </c>
       <c r="K59">
         <f t="shared" si="17"/>
-        <v>1.2776575276575277E-2</v>
+        <v>1.2246426924850161E-2</v>
       </c>
       <c r="L59">
         <f t="shared" si="16"/>
-        <v>0.76659451659451661</v>
+        <v>0.73478561549100974</v>
       </c>
       <c r="M59">
         <f t="shared" si="6"/>
-        <v>45.995670995670999</v>
+        <v>44.087136929460584</v>
       </c>
       <c r="N59">
         <f t="shared" si="7"/>
-        <v>367.96536796536799</v>
+        <v>352.69709543568467</v>
       </c>
       <c r="O59">
         <f t="shared" si="8"/>
@@ -3190,19 +3190,19 @@
       </c>
       <c r="K60">
         <f t="shared" si="17"/>
-        <v>1.3528138528138528E-2</v>
+        <v>1.2966804979253113E-2</v>
       </c>
       <c r="L60">
         <f t="shared" si="16"/>
-        <v>0.81168831168831168</v>
+        <v>0.77800829875518673</v>
       </c>
       <c r="M60">
         <f t="shared" si="6"/>
-        <v>48.701298701298704</v>
+        <v>46.680497925311201</v>
       </c>
       <c r="N60">
         <f t="shared" si="7"/>
-        <v>389.61038961038963</v>
+        <v>373.44398340248961</v>
       </c>
       <c r="O60">
         <f t="shared" si="8"/>
@@ -3243,19 +3243,19 @@
       </c>
       <c r="K61">
         <f t="shared" si="17"/>
-        <v>1.4279701779701779E-2</v>
+        <v>1.3687183033656063E-2</v>
       </c>
       <c r="L61">
         <f t="shared" si="16"/>
-        <v>0.85678210678210676</v>
+        <v>0.82123098201936373</v>
       </c>
       <c r="M61">
         <f t="shared" si="6"/>
-        <v>51.406926406926409</v>
+        <v>49.273858921161825</v>
       </c>
       <c r="N61">
         <f t="shared" si="7"/>
-        <v>411.25541125541127</v>
+        <v>394.1908713692946</v>
       </c>
       <c r="O61">
         <f t="shared" si="8"/>
@@ -3296,19 +3296,19 @@
       </c>
       <c r="K62">
         <f t="shared" si="17"/>
-        <v>1.5031265031265031E-2</v>
+        <v>1.4407561088059014E-2</v>
       </c>
       <c r="L62">
         <f t="shared" si="16"/>
-        <v>0.90187590187590183</v>
+        <v>0.86445366528354084</v>
       </c>
       <c r="M62">
         <f t="shared" si="6"/>
-        <v>54.112554112554115</v>
+        <v>51.867219917012449</v>
       </c>
       <c r="N62">
         <f t="shared" si="7"/>
-        <v>432.90043290043292</v>
+        <v>414.93775933609959</v>
       </c>
       <c r="O62">
         <f t="shared" si="8"/>
@@ -3317,6 +3317,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="J16:N16"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="D37:J37"/>
     <mergeCell ref="K37:Q37"/>
     <mergeCell ref="C5:D5"/>
@@ -3326,14 +3334,6 @@
     <mergeCell ref="C27:I27"/>
     <mergeCell ref="J27:N27"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="J16:N16"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C14:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>